<commit_message>
add sedi to parameters excel
</commit_message>
<xml_diff>
--- a/coral_data_and_custom_parameters.xlsx
+++ b/coral_data_and_custom_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10908"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katyaovsyanikova/Documents/GitHub/Coral-Model/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uq-my.sharepoint.com/personal/uqrbutto_uq_edu_au/Documents/PhD_proj_pollution_on_coral_reefs/Coral-Model-Rio_sediment_extension/Coral-Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32B717CB-20CE-4090-85C7-148C11B2FA28}"/>
   <bookViews>
-    <workbookView xWindow="29700" yWindow="500" windowWidth="36860" windowHeight="18360" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-4290" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Real_Cover" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Growth_Rates" sheetId="5" r:id="rId5"/>
     <sheet name="DHW_Years" sheetId="6" r:id="rId6"/>
     <sheet name="Cyclone_Years" sheetId="7" r:id="rId7"/>
+    <sheet name="Sediment_Exposure" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
   <si>
     <t>Year</t>
   </si>
@@ -97,12 +98,21 @@
   <si>
     <t>Distance_km</t>
   </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Suspended_sediment</t>
+  </si>
+  <si>
+    <t>Deposited_sediment</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -118,6 +128,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -127,7 +152,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -150,15 +175,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,14 +509,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -485,7 +530,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2000</v>
       </c>
@@ -499,7 +544,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2001</v>
       </c>
@@ -513,7 +558,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2002</v>
       </c>
@@ -527,7 +572,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2003</v>
       </c>
@@ -541,7 +586,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2004</v>
       </c>
@@ -555,7 +600,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2005</v>
       </c>
@@ -569,7 +614,7 @@
         <v>15.2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2006</v>
       </c>
@@ -583,7 +628,7 @@
         <v>14.1</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2007</v>
       </c>
@@ -597,7 +642,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2008</v>
       </c>
@@ -611,7 +656,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2009</v>
       </c>
@@ -625,7 +670,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2010</v>
       </c>
@@ -639,7 +684,7 @@
         <v>13.9</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2011</v>
       </c>
@@ -661,9 +706,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -677,7 +722,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>5</v>
       </c>
@@ -691,7 +736,7 @@
         <v>7.8</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>10</v>
       </c>
@@ -705,7 +750,7 @@
         <v>10.1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>15</v>
       </c>
@@ -719,7 +764,7 @@
         <v>23.4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>20</v>
       </c>
@@ -733,7 +778,7 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>25</v>
       </c>
@@ -747,7 +792,7 @@
         <v>9.6999999999999993</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>30</v>
       </c>
@@ -761,7 +806,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>35</v>
       </c>
@@ -775,7 +820,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>40</v>
       </c>
@@ -789,7 +834,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>45</v>
       </c>
@@ -803,7 +848,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>50</v>
       </c>
@@ -817,7 +862,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>55</v>
       </c>
@@ -831,7 +876,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>60</v>
       </c>
@@ -845,7 +890,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>65</v>
       </c>
@@ -859,7 +904,7 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>70</v>
       </c>
@@ -873,7 +918,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>75</v>
       </c>
@@ -887,7 +932,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>80</v>
       </c>
@@ -901,7 +946,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>85</v>
       </c>
@@ -915,7 +960,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>90</v>
       </c>
@@ -929,7 +974,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>95</v>
       </c>
@@ -943,7 +988,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>100</v>
       </c>
@@ -965,12 +1010,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -984,7 +1029,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>5</v>
       </c>
@@ -998,7 +1043,7 @@
         <v>1.17E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>10</v>
       </c>
@@ -1012,7 +1057,7 @@
         <v>1.3599999999999999E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>15</v>
       </c>
@@ -1026,7 +1071,7 @@
         <v>1.5599999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>20</v>
       </c>
@@ -1040,7 +1085,7 @@
         <v>1.7600000000000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>25</v>
       </c>
@@ -1054,7 +1099,7 @@
         <v>1.9599999999999999E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>30</v>
       </c>
@@ -1068,7 +1113,7 @@
         <v>2.1600000000000001E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>35</v>
       </c>
@@ -1082,7 +1127,7 @@
         <v>2.3599999999999999E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>40</v>
       </c>
@@ -1096,7 +1141,7 @@
         <v>2.5600000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>45</v>
       </c>
@@ -1110,7 +1155,7 @@
         <v>2.76E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>50</v>
       </c>
@@ -1124,7 +1169,7 @@
         <v>2.9600000000000001E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>55</v>
       </c>
@@ -1138,7 +1183,7 @@
         <v>3.1600000000000003E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>60</v>
       </c>
@@ -1152,7 +1197,7 @@
         <v>3.3500000000000002E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>65</v>
       </c>
@@ -1166,7 +1211,7 @@
         <v>3.5499999999999997E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>70</v>
       </c>
@@ -1180,7 +1225,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>75</v>
       </c>
@@ -1194,7 +1239,7 @@
         <v>3.95E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>80</v>
       </c>
@@ -1208,7 +1253,7 @@
         <v>4.1500000000000002E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>85</v>
       </c>
@@ -1222,7 +1267,7 @@
         <v>4.3499999999999997E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>90</v>
       </c>
@@ -1236,7 +1281,7 @@
         <v>4.5499999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>95</v>
       </c>
@@ -1250,7 +1295,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>100</v>
       </c>
@@ -1272,9 +1317,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1288,7 +1333,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>5</v>
       </c>
@@ -1302,7 +1347,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>10</v>
       </c>
@@ -1316,7 +1361,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>15</v>
       </c>
@@ -1330,7 +1375,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>20</v>
       </c>
@@ -1344,7 +1389,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>25</v>
       </c>
@@ -1358,7 +1403,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>30</v>
       </c>
@@ -1372,7 +1417,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>35</v>
       </c>
@@ -1386,7 +1431,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>40</v>
       </c>
@@ -1400,7 +1445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>45</v>
       </c>
@@ -1414,7 +1459,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>50</v>
       </c>
@@ -1428,7 +1473,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>55</v>
       </c>
@@ -1442,7 +1487,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>60</v>
       </c>
@@ -1456,7 +1501,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>65</v>
       </c>
@@ -1470,7 +1515,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>70</v>
       </c>
@@ -1484,7 +1529,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>75</v>
       </c>
@@ -1498,7 +1543,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>80</v>
       </c>
@@ -1512,7 +1557,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>85</v>
       </c>
@@ -1526,7 +1571,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>90</v>
       </c>
@@ -1540,7 +1585,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>95</v>
       </c>
@@ -1554,7 +1599,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>100</v>
       </c>
@@ -1576,9 +1621,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -1586,7 +1631,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1594,7 +1639,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1602,7 +1647,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1618,9 +1663,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1628,7 +1673,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2013</v>
       </c>
@@ -1636,7 +1681,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2016</v>
       </c>
@@ -1644,7 +1689,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2018</v>
       </c>
@@ -1652,7 +1697,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2020</v>
       </c>
@@ -1668,9 +1713,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1681,7 +1726,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2001</v>
       </c>
@@ -1692,7 +1737,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2007</v>
       </c>
@@ -1701,6 +1746,3390 @@
       </c>
       <c r="C3">
         <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E132077E-EAF7-4017-9CD9-9B94D708D64A}">
+  <dimension ref="A1:D241"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4">
+        <v>5</v>
+      </c>
+      <c r="D2" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2</v>
+      </c>
+      <c r="C3" s="4">
+        <v>5</v>
+      </c>
+      <c r="D3" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4">
+        <v>5</v>
+      </c>
+      <c r="D4" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B5" s="4">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B6" s="4">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4">
+        <v>5</v>
+      </c>
+      <c r="D6" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B7" s="4">
+        <v>6</v>
+      </c>
+      <c r="C7" s="4">
+        <v>5</v>
+      </c>
+      <c r="D7" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B8" s="4">
+        <v>7</v>
+      </c>
+      <c r="C8" s="4">
+        <v>5</v>
+      </c>
+      <c r="D8" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B9" s="4">
+        <v>8</v>
+      </c>
+      <c r="C9" s="4">
+        <v>5</v>
+      </c>
+      <c r="D9" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B10" s="4">
+        <v>9</v>
+      </c>
+      <c r="C10" s="4">
+        <v>5</v>
+      </c>
+      <c r="D10" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B11" s="4">
+        <v>10</v>
+      </c>
+      <c r="C11" s="4">
+        <v>5</v>
+      </c>
+      <c r="D11" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B12" s="4">
+        <v>11</v>
+      </c>
+      <c r="C12" s="4">
+        <v>5</v>
+      </c>
+      <c r="D12" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>2005</v>
+      </c>
+      <c r="B13" s="4">
+        <v>12</v>
+      </c>
+      <c r="C13" s="4">
+        <v>5</v>
+      </c>
+      <c r="D13" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B14" s="4">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4">
+        <v>20</v>
+      </c>
+      <c r="D14" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B15" s="4">
+        <v>2</v>
+      </c>
+      <c r="C15" s="4">
+        <v>20</v>
+      </c>
+      <c r="D15" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B16" s="4">
+        <v>3</v>
+      </c>
+      <c r="C16" s="4">
+        <v>20</v>
+      </c>
+      <c r="D16" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B17" s="4">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4">
+        <v>20</v>
+      </c>
+      <c r="D17" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B18" s="4">
+        <v>5</v>
+      </c>
+      <c r="C18" s="4">
+        <v>20</v>
+      </c>
+      <c r="D18" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B19" s="4">
+        <v>6</v>
+      </c>
+      <c r="C19" s="4">
+        <v>20</v>
+      </c>
+      <c r="D19" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B20" s="4">
+        <v>7</v>
+      </c>
+      <c r="C20" s="4">
+        <v>20</v>
+      </c>
+      <c r="D20" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B21" s="4">
+        <v>8</v>
+      </c>
+      <c r="C21" s="4">
+        <v>20</v>
+      </c>
+      <c r="D21" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B22" s="4">
+        <v>9</v>
+      </c>
+      <c r="C22" s="4">
+        <v>20</v>
+      </c>
+      <c r="D22" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B23" s="4">
+        <v>10</v>
+      </c>
+      <c r="C23" s="4">
+        <v>20</v>
+      </c>
+      <c r="D23" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B24" s="4">
+        <v>11</v>
+      </c>
+      <c r="C24" s="4">
+        <v>20</v>
+      </c>
+      <c r="D24" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
+        <v>2006</v>
+      </c>
+      <c r="B25" s="4">
+        <v>12</v>
+      </c>
+      <c r="C25" s="4">
+        <v>20</v>
+      </c>
+      <c r="D25" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B26" s="4">
+        <v>1</v>
+      </c>
+      <c r="C26" s="4">
+        <v>5</v>
+      </c>
+      <c r="D26" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B27" s="4">
+        <v>2</v>
+      </c>
+      <c r="C27" s="4">
+        <v>5</v>
+      </c>
+      <c r="D27" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B28" s="4">
+        <v>3</v>
+      </c>
+      <c r="C28" s="4">
+        <v>5</v>
+      </c>
+      <c r="D28" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B29" s="4">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4">
+        <v>5</v>
+      </c>
+      <c r="D29" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B30" s="4">
+        <v>5</v>
+      </c>
+      <c r="C30" s="4">
+        <v>5</v>
+      </c>
+      <c r="D30" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B31" s="4">
+        <v>6</v>
+      </c>
+      <c r="C31" s="4">
+        <v>5</v>
+      </c>
+      <c r="D31" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B32" s="4">
+        <v>7</v>
+      </c>
+      <c r="C32" s="4">
+        <v>5</v>
+      </c>
+      <c r="D32" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B33" s="4">
+        <v>8</v>
+      </c>
+      <c r="C33" s="4">
+        <v>5</v>
+      </c>
+      <c r="D33" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B34" s="4">
+        <v>9</v>
+      </c>
+      <c r="C34" s="4">
+        <v>5</v>
+      </c>
+      <c r="D34" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B35" s="4">
+        <v>10</v>
+      </c>
+      <c r="C35" s="4">
+        <v>5</v>
+      </c>
+      <c r="D35" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B36" s="4">
+        <v>11</v>
+      </c>
+      <c r="C36" s="4">
+        <v>5</v>
+      </c>
+      <c r="D36" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" s="4">
+        <v>2007</v>
+      </c>
+      <c r="B37" s="4">
+        <v>12</v>
+      </c>
+      <c r="C37" s="4">
+        <v>5</v>
+      </c>
+      <c r="D37" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B38" s="4">
+        <v>1</v>
+      </c>
+      <c r="C38" s="4">
+        <v>5</v>
+      </c>
+      <c r="D38" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B39" s="4">
+        <v>2</v>
+      </c>
+      <c r="C39" s="4">
+        <v>5</v>
+      </c>
+      <c r="D39" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B40" s="4">
+        <v>3</v>
+      </c>
+      <c r="C40" s="4">
+        <v>5</v>
+      </c>
+      <c r="D40" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B41" s="4">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4">
+        <v>5</v>
+      </c>
+      <c r="D41" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B42" s="4">
+        <v>5</v>
+      </c>
+      <c r="C42" s="4">
+        <v>5</v>
+      </c>
+      <c r="D42" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B43" s="4">
+        <v>6</v>
+      </c>
+      <c r="C43" s="4">
+        <v>5</v>
+      </c>
+      <c r="D43" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B44" s="4">
+        <v>7</v>
+      </c>
+      <c r="C44" s="4">
+        <v>5</v>
+      </c>
+      <c r="D44" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B45" s="4">
+        <v>8</v>
+      </c>
+      <c r="C45" s="4">
+        <v>5</v>
+      </c>
+      <c r="D45" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B46" s="4">
+        <v>9</v>
+      </c>
+      <c r="C46" s="4">
+        <v>5</v>
+      </c>
+      <c r="D46" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B47" s="4">
+        <v>10</v>
+      </c>
+      <c r="C47" s="4">
+        <v>5</v>
+      </c>
+      <c r="D47" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B48" s="4">
+        <v>11</v>
+      </c>
+      <c r="C48" s="4">
+        <v>5</v>
+      </c>
+      <c r="D48" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" s="4">
+        <v>2008</v>
+      </c>
+      <c r="B49" s="4">
+        <v>12</v>
+      </c>
+      <c r="C49" s="4">
+        <v>5</v>
+      </c>
+      <c r="D49" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B50" s="4">
+        <v>1</v>
+      </c>
+      <c r="C50" s="4">
+        <v>5</v>
+      </c>
+      <c r="D50" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B51" s="4">
+        <v>2</v>
+      </c>
+      <c r="C51" s="4">
+        <v>5</v>
+      </c>
+      <c r="D51" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B52" s="4">
+        <v>3</v>
+      </c>
+      <c r="C52" s="4">
+        <v>5</v>
+      </c>
+      <c r="D52" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B53" s="4">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4">
+        <v>5</v>
+      </c>
+      <c r="D53" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B54" s="4">
+        <v>5</v>
+      </c>
+      <c r="C54" s="4">
+        <v>5</v>
+      </c>
+      <c r="D54" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B55" s="4">
+        <v>6</v>
+      </c>
+      <c r="C55" s="4">
+        <v>5</v>
+      </c>
+      <c r="D55" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B56" s="4">
+        <v>7</v>
+      </c>
+      <c r="C56" s="4">
+        <v>5</v>
+      </c>
+      <c r="D56" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B57" s="4">
+        <v>8</v>
+      </c>
+      <c r="C57" s="4">
+        <v>5</v>
+      </c>
+      <c r="D57" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B58" s="4">
+        <v>9</v>
+      </c>
+      <c r="C58" s="4">
+        <v>5</v>
+      </c>
+      <c r="D58" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B59" s="4">
+        <v>10</v>
+      </c>
+      <c r="C59" s="4">
+        <v>5</v>
+      </c>
+      <c r="D59" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B60" s="4">
+        <v>11</v>
+      </c>
+      <c r="C60" s="4">
+        <v>5</v>
+      </c>
+      <c r="D60" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" s="4">
+        <v>2009</v>
+      </c>
+      <c r="B61" s="4">
+        <v>12</v>
+      </c>
+      <c r="C61" s="4">
+        <v>5</v>
+      </c>
+      <c r="D61" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B62" s="4">
+        <v>1</v>
+      </c>
+      <c r="C62" s="4">
+        <v>5</v>
+      </c>
+      <c r="D62" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B63" s="4">
+        <v>2</v>
+      </c>
+      <c r="C63" s="4">
+        <v>5</v>
+      </c>
+      <c r="D63" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B64" s="4">
+        <v>3</v>
+      </c>
+      <c r="C64" s="4">
+        <v>5</v>
+      </c>
+      <c r="D64" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B65" s="4">
+        <v>4</v>
+      </c>
+      <c r="C65" s="4">
+        <v>5</v>
+      </c>
+      <c r="D65" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B66" s="4">
+        <v>5</v>
+      </c>
+      <c r="C66" s="4">
+        <v>5</v>
+      </c>
+      <c r="D66" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B67" s="4">
+        <v>6</v>
+      </c>
+      <c r="C67" s="4">
+        <v>5</v>
+      </c>
+      <c r="D67" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B68" s="4">
+        <v>7</v>
+      </c>
+      <c r="C68" s="4">
+        <v>5</v>
+      </c>
+      <c r="D68" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B69" s="4">
+        <v>8</v>
+      </c>
+      <c r="C69" s="4">
+        <v>5</v>
+      </c>
+      <c r="D69" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B70" s="4">
+        <v>9</v>
+      </c>
+      <c r="C70" s="4">
+        <v>5</v>
+      </c>
+      <c r="D70" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B71" s="4">
+        <v>10</v>
+      </c>
+      <c r="C71" s="4">
+        <v>5</v>
+      </c>
+      <c r="D71" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B72" s="4">
+        <v>11</v>
+      </c>
+      <c r="C72" s="4">
+        <v>5</v>
+      </c>
+      <c r="D72" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" s="4">
+        <v>2010</v>
+      </c>
+      <c r="B73" s="4">
+        <v>12</v>
+      </c>
+      <c r="C73" s="4">
+        <v>5</v>
+      </c>
+      <c r="D73" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B74" s="4">
+        <v>1</v>
+      </c>
+      <c r="C74" s="4">
+        <v>5</v>
+      </c>
+      <c r="D74" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B75" s="4">
+        <v>2</v>
+      </c>
+      <c r="C75" s="4">
+        <v>5</v>
+      </c>
+      <c r="D75" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B76" s="4">
+        <v>3</v>
+      </c>
+      <c r="C76" s="4">
+        <v>5</v>
+      </c>
+      <c r="D76" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B77" s="4">
+        <v>4</v>
+      </c>
+      <c r="C77" s="4">
+        <v>5</v>
+      </c>
+      <c r="D77" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B78" s="4">
+        <v>5</v>
+      </c>
+      <c r="C78" s="4">
+        <v>5</v>
+      </c>
+      <c r="D78" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B79" s="4">
+        <v>6</v>
+      </c>
+      <c r="C79" s="4">
+        <v>5</v>
+      </c>
+      <c r="D79" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B80" s="4">
+        <v>7</v>
+      </c>
+      <c r="C80" s="4">
+        <v>5</v>
+      </c>
+      <c r="D80" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B81" s="4">
+        <v>8</v>
+      </c>
+      <c r="C81" s="4">
+        <v>5</v>
+      </c>
+      <c r="D81" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B82" s="4">
+        <v>9</v>
+      </c>
+      <c r="C82" s="4">
+        <v>5</v>
+      </c>
+      <c r="D82" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B83" s="4">
+        <v>10</v>
+      </c>
+      <c r="C83" s="4">
+        <v>5</v>
+      </c>
+      <c r="D83" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B84" s="4">
+        <v>11</v>
+      </c>
+      <c r="C84" s="4">
+        <v>5</v>
+      </c>
+      <c r="D84" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" s="4">
+        <v>2011</v>
+      </c>
+      <c r="B85" s="4">
+        <v>12</v>
+      </c>
+      <c r="C85" s="4">
+        <v>5</v>
+      </c>
+      <c r="D85" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B86" s="4">
+        <v>1</v>
+      </c>
+      <c r="C86" s="4">
+        <v>5</v>
+      </c>
+      <c r="D86" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B87" s="4">
+        <v>2</v>
+      </c>
+      <c r="C87" s="4">
+        <v>5</v>
+      </c>
+      <c r="D87" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B88" s="4">
+        <v>3</v>
+      </c>
+      <c r="C88" s="4">
+        <v>5</v>
+      </c>
+      <c r="D88" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B89" s="4">
+        <v>4</v>
+      </c>
+      <c r="C89" s="4">
+        <v>5</v>
+      </c>
+      <c r="D89" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B90" s="4">
+        <v>5</v>
+      </c>
+      <c r="C90" s="4">
+        <v>5</v>
+      </c>
+      <c r="D90" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B91" s="4">
+        <v>6</v>
+      </c>
+      <c r="C91" s="4">
+        <v>5</v>
+      </c>
+      <c r="D91" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B92" s="4">
+        <v>7</v>
+      </c>
+      <c r="C92" s="4">
+        <v>5</v>
+      </c>
+      <c r="D92" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B93" s="4">
+        <v>8</v>
+      </c>
+      <c r="C93" s="4">
+        <v>5</v>
+      </c>
+      <c r="D93" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B94" s="4">
+        <v>9</v>
+      </c>
+      <c r="C94" s="4">
+        <v>5</v>
+      </c>
+      <c r="D94" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B95" s="4">
+        <v>10</v>
+      </c>
+      <c r="C95" s="4">
+        <v>5</v>
+      </c>
+      <c r="D95" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B96" s="4">
+        <v>11</v>
+      </c>
+      <c r="C96" s="4">
+        <v>5</v>
+      </c>
+      <c r="D96" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B97" s="4">
+        <v>12</v>
+      </c>
+      <c r="C97" s="4">
+        <v>5</v>
+      </c>
+      <c r="D97" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B98" s="4">
+        <v>1</v>
+      </c>
+      <c r="C98" s="4">
+        <v>5</v>
+      </c>
+      <c r="D98" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B99" s="4">
+        <v>2</v>
+      </c>
+      <c r="C99" s="4">
+        <v>5</v>
+      </c>
+      <c r="D99" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B100" s="4">
+        <v>3</v>
+      </c>
+      <c r="C100" s="4">
+        <v>5</v>
+      </c>
+      <c r="D100" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B101" s="4">
+        <v>4</v>
+      </c>
+      <c r="C101" s="4">
+        <v>5</v>
+      </c>
+      <c r="D101" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B102" s="4">
+        <v>5</v>
+      </c>
+      <c r="C102" s="4">
+        <v>5</v>
+      </c>
+      <c r="D102" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B103" s="4">
+        <v>6</v>
+      </c>
+      <c r="C103" s="4">
+        <v>5</v>
+      </c>
+      <c r="D103" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B104" s="4">
+        <v>7</v>
+      </c>
+      <c r="C104" s="4">
+        <v>5</v>
+      </c>
+      <c r="D104" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B105" s="4">
+        <v>8</v>
+      </c>
+      <c r="C105" s="4">
+        <v>5</v>
+      </c>
+      <c r="D105" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B106" s="4">
+        <v>9</v>
+      </c>
+      <c r="C106" s="4">
+        <v>5</v>
+      </c>
+      <c r="D106" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B107" s="4">
+        <v>10</v>
+      </c>
+      <c r="C107" s="4">
+        <v>5</v>
+      </c>
+      <c r="D107" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B108" s="4">
+        <v>11</v>
+      </c>
+      <c r="C108" s="4">
+        <v>5</v>
+      </c>
+      <c r="D108" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B109" s="4">
+        <v>12</v>
+      </c>
+      <c r="C109" s="4">
+        <v>5</v>
+      </c>
+      <c r="D109" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B110" s="4">
+        <v>1</v>
+      </c>
+      <c r="C110" s="4">
+        <v>5</v>
+      </c>
+      <c r="D110" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B111" s="4">
+        <v>2</v>
+      </c>
+      <c r="C111" s="4">
+        <v>5</v>
+      </c>
+      <c r="D111" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B112" s="4">
+        <v>3</v>
+      </c>
+      <c r="C112" s="4">
+        <v>5</v>
+      </c>
+      <c r="D112" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B113" s="4">
+        <v>4</v>
+      </c>
+      <c r="C113" s="4">
+        <v>5</v>
+      </c>
+      <c r="D113" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B114" s="4">
+        <v>5</v>
+      </c>
+      <c r="C114" s="4">
+        <v>5</v>
+      </c>
+      <c r="D114" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B115" s="4">
+        <v>6</v>
+      </c>
+      <c r="C115" s="4">
+        <v>5</v>
+      </c>
+      <c r="D115" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B116" s="4">
+        <v>7</v>
+      </c>
+      <c r="C116" s="4">
+        <v>5</v>
+      </c>
+      <c r="D116" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B117" s="4">
+        <v>8</v>
+      </c>
+      <c r="C117" s="4">
+        <v>5</v>
+      </c>
+      <c r="D117" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B118" s="4">
+        <v>9</v>
+      </c>
+      <c r="C118" s="4">
+        <v>5</v>
+      </c>
+      <c r="D118" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B119" s="4">
+        <v>10</v>
+      </c>
+      <c r="C119" s="4">
+        <v>5</v>
+      </c>
+      <c r="D119" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A120" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B120" s="4">
+        <v>11</v>
+      </c>
+      <c r="C120" s="4">
+        <v>5</v>
+      </c>
+      <c r="D120" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A121" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B121" s="4">
+        <v>12</v>
+      </c>
+      <c r="C121" s="4">
+        <v>5</v>
+      </c>
+      <c r="D121" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A122" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B122" s="4">
+        <v>1</v>
+      </c>
+      <c r="C122" s="4">
+        <v>5</v>
+      </c>
+      <c r="D122" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B123" s="4">
+        <v>2</v>
+      </c>
+      <c r="C123" s="4">
+        <v>5</v>
+      </c>
+      <c r="D123" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B124" s="4">
+        <v>3</v>
+      </c>
+      <c r="C124" s="4">
+        <v>5</v>
+      </c>
+      <c r="D124" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B125" s="4">
+        <v>4</v>
+      </c>
+      <c r="C125" s="4">
+        <v>5</v>
+      </c>
+      <c r="D125" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B126" s="4">
+        <v>5</v>
+      </c>
+      <c r="C126" s="4">
+        <v>5</v>
+      </c>
+      <c r="D126" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B127" s="4">
+        <v>6</v>
+      </c>
+      <c r="C127" s="4">
+        <v>5</v>
+      </c>
+      <c r="D127" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B128" s="4">
+        <v>7</v>
+      </c>
+      <c r="C128" s="4">
+        <v>5</v>
+      </c>
+      <c r="D128" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B129" s="4">
+        <v>8</v>
+      </c>
+      <c r="C129" s="4">
+        <v>5</v>
+      </c>
+      <c r="D129" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B130" s="4">
+        <v>9</v>
+      </c>
+      <c r="C130" s="4">
+        <v>5</v>
+      </c>
+      <c r="D130" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B131" s="4">
+        <v>10</v>
+      </c>
+      <c r="C131" s="4">
+        <v>5</v>
+      </c>
+      <c r="D131" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A132" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B132" s="4">
+        <v>11</v>
+      </c>
+      <c r="C132" s="4">
+        <v>5</v>
+      </c>
+      <c r="D132" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B133" s="4">
+        <v>12</v>
+      </c>
+      <c r="C133" s="4">
+        <v>5</v>
+      </c>
+      <c r="D133" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A134" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B134" s="4">
+        <v>1</v>
+      </c>
+      <c r="C134" s="4">
+        <v>5</v>
+      </c>
+      <c r="D134" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A135" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B135" s="4">
+        <v>2</v>
+      </c>
+      <c r="C135" s="4">
+        <v>5</v>
+      </c>
+      <c r="D135" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A136" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B136" s="4">
+        <v>3</v>
+      </c>
+      <c r="C136" s="4">
+        <v>5</v>
+      </c>
+      <c r="D136" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A137" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B137" s="4">
+        <v>4</v>
+      </c>
+      <c r="C137" s="4">
+        <v>5</v>
+      </c>
+      <c r="D137" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A138" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B138" s="4">
+        <v>5</v>
+      </c>
+      <c r="C138" s="4">
+        <v>5</v>
+      </c>
+      <c r="D138" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A139" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B139" s="4">
+        <v>6</v>
+      </c>
+      <c r="C139" s="4">
+        <v>5</v>
+      </c>
+      <c r="D139" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A140" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B140" s="4">
+        <v>7</v>
+      </c>
+      <c r="C140" s="4">
+        <v>5</v>
+      </c>
+      <c r="D140" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A141" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B141" s="4">
+        <v>8</v>
+      </c>
+      <c r="C141" s="4">
+        <v>5</v>
+      </c>
+      <c r="D141" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A142" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B142" s="4">
+        <v>9</v>
+      </c>
+      <c r="C142" s="4">
+        <v>5</v>
+      </c>
+      <c r="D142" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A143" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B143" s="4">
+        <v>10</v>
+      </c>
+      <c r="C143" s="4">
+        <v>5</v>
+      </c>
+      <c r="D143" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A144" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B144" s="4">
+        <v>11</v>
+      </c>
+      <c r="C144" s="4">
+        <v>5</v>
+      </c>
+      <c r="D144" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A145" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B145" s="4">
+        <v>12</v>
+      </c>
+      <c r="C145" s="4">
+        <v>5</v>
+      </c>
+      <c r="D145" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A146" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B146" s="4">
+        <v>1</v>
+      </c>
+      <c r="C146" s="4">
+        <v>5</v>
+      </c>
+      <c r="D146" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A147" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B147" s="4">
+        <v>2</v>
+      </c>
+      <c r="C147" s="4">
+        <v>5</v>
+      </c>
+      <c r="D147" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A148" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B148" s="4">
+        <v>3</v>
+      </c>
+      <c r="C148" s="4">
+        <v>5</v>
+      </c>
+      <c r="D148" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A149" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B149" s="4">
+        <v>4</v>
+      </c>
+      <c r="C149" s="4">
+        <v>5</v>
+      </c>
+      <c r="D149" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A150" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B150" s="4">
+        <v>5</v>
+      </c>
+      <c r="C150" s="4">
+        <v>5</v>
+      </c>
+      <c r="D150" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A151" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B151" s="4">
+        <v>6</v>
+      </c>
+      <c r="C151" s="4">
+        <v>5</v>
+      </c>
+      <c r="D151" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A152" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B152" s="4">
+        <v>7</v>
+      </c>
+      <c r="C152" s="4">
+        <v>5</v>
+      </c>
+      <c r="D152" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A153" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B153" s="4">
+        <v>8</v>
+      </c>
+      <c r="C153" s="4">
+        <v>5</v>
+      </c>
+      <c r="D153" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A154" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B154" s="4">
+        <v>9</v>
+      </c>
+      <c r="C154" s="4">
+        <v>5</v>
+      </c>
+      <c r="D154" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A155" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B155" s="4">
+        <v>10</v>
+      </c>
+      <c r="C155" s="4">
+        <v>5</v>
+      </c>
+      <c r="D155" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A156" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B156" s="4">
+        <v>11</v>
+      </c>
+      <c r="C156" s="4">
+        <v>5</v>
+      </c>
+      <c r="D156" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A157" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B157" s="4">
+        <v>12</v>
+      </c>
+      <c r="C157" s="4">
+        <v>5</v>
+      </c>
+      <c r="D157" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A158" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B158" s="4">
+        <v>1</v>
+      </c>
+      <c r="C158" s="4">
+        <v>5</v>
+      </c>
+      <c r="D158" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A159" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B159" s="4">
+        <v>2</v>
+      </c>
+      <c r="C159" s="4">
+        <v>5</v>
+      </c>
+      <c r="D159" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A160" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B160" s="4">
+        <v>3</v>
+      </c>
+      <c r="C160" s="4">
+        <v>5</v>
+      </c>
+      <c r="D160" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A161" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B161" s="4">
+        <v>4</v>
+      </c>
+      <c r="C161" s="4">
+        <v>5</v>
+      </c>
+      <c r="D161" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A162" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B162" s="4">
+        <v>5</v>
+      </c>
+      <c r="C162" s="4">
+        <v>5</v>
+      </c>
+      <c r="D162" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A163" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B163" s="4">
+        <v>6</v>
+      </c>
+      <c r="C163" s="4">
+        <v>5</v>
+      </c>
+      <c r="D163" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A164" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B164" s="4">
+        <v>7</v>
+      </c>
+      <c r="C164" s="4">
+        <v>5</v>
+      </c>
+      <c r="D164" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A165" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B165" s="4">
+        <v>8</v>
+      </c>
+      <c r="C165" s="4">
+        <v>5</v>
+      </c>
+      <c r="D165" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A166" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B166" s="4">
+        <v>9</v>
+      </c>
+      <c r="C166" s="4">
+        <v>5</v>
+      </c>
+      <c r="D166" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A167" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B167" s="4">
+        <v>10</v>
+      </c>
+      <c r="C167" s="4">
+        <v>5</v>
+      </c>
+      <c r="D167" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A168" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B168" s="4">
+        <v>11</v>
+      </c>
+      <c r="C168" s="4">
+        <v>5</v>
+      </c>
+      <c r="D168" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A169" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B169" s="4">
+        <v>12</v>
+      </c>
+      <c r="C169" s="4">
+        <v>5</v>
+      </c>
+      <c r="D169" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A170" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B170" s="4">
+        <v>1</v>
+      </c>
+      <c r="C170" s="4">
+        <v>5</v>
+      </c>
+      <c r="D170" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A171" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B171" s="4">
+        <v>2</v>
+      </c>
+      <c r="C171" s="4">
+        <v>5</v>
+      </c>
+      <c r="D171" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A172" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B172" s="4">
+        <v>3</v>
+      </c>
+      <c r="C172" s="4">
+        <v>5</v>
+      </c>
+      <c r="D172" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A173" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B173" s="4">
+        <v>4</v>
+      </c>
+      <c r="C173" s="4">
+        <v>5</v>
+      </c>
+      <c r="D173" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A174" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B174" s="4">
+        <v>5</v>
+      </c>
+      <c r="C174" s="4">
+        <v>5</v>
+      </c>
+      <c r="D174" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A175" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B175" s="4">
+        <v>6</v>
+      </c>
+      <c r="C175" s="4">
+        <v>5</v>
+      </c>
+      <c r="D175" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A176" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B176" s="4">
+        <v>7</v>
+      </c>
+      <c r="C176" s="4">
+        <v>5</v>
+      </c>
+      <c r="D176" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A177" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B177" s="4">
+        <v>8</v>
+      </c>
+      <c r="C177" s="4">
+        <v>5</v>
+      </c>
+      <c r="D177" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A178" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B178" s="4">
+        <v>9</v>
+      </c>
+      <c r="C178" s="4">
+        <v>5</v>
+      </c>
+      <c r="D178" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A179" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B179" s="4">
+        <v>10</v>
+      </c>
+      <c r="C179" s="4">
+        <v>5</v>
+      </c>
+      <c r="D179" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A180" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B180" s="4">
+        <v>11</v>
+      </c>
+      <c r="C180" s="4">
+        <v>5</v>
+      </c>
+      <c r="D180" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A181" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B181" s="4">
+        <v>12</v>
+      </c>
+      <c r="C181" s="4">
+        <v>5</v>
+      </c>
+      <c r="D181" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A182" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B182" s="4">
+        <v>1</v>
+      </c>
+      <c r="C182" s="4">
+        <v>5</v>
+      </c>
+      <c r="D182" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A183" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B183" s="4">
+        <v>2</v>
+      </c>
+      <c r="C183" s="4">
+        <v>5</v>
+      </c>
+      <c r="D183" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A184" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B184" s="4">
+        <v>3</v>
+      </c>
+      <c r="C184" s="4">
+        <v>5</v>
+      </c>
+      <c r="D184" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A185" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B185" s="4">
+        <v>4</v>
+      </c>
+      <c r="C185" s="4">
+        <v>5</v>
+      </c>
+      <c r="D185" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A186" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B186" s="4">
+        <v>5</v>
+      </c>
+      <c r="C186" s="4">
+        <v>5</v>
+      </c>
+      <c r="D186" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A187" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B187" s="4">
+        <v>6</v>
+      </c>
+      <c r="C187" s="4">
+        <v>5</v>
+      </c>
+      <c r="D187" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A188" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B188" s="4">
+        <v>7</v>
+      </c>
+      <c r="C188" s="4">
+        <v>5</v>
+      </c>
+      <c r="D188" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A189" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B189" s="4">
+        <v>8</v>
+      </c>
+      <c r="C189" s="4">
+        <v>5</v>
+      </c>
+      <c r="D189" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A190" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B190" s="4">
+        <v>9</v>
+      </c>
+      <c r="C190" s="4">
+        <v>5</v>
+      </c>
+      <c r="D190" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A191" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B191" s="4">
+        <v>10</v>
+      </c>
+      <c r="C191" s="4">
+        <v>5</v>
+      </c>
+      <c r="D191" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A192" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B192" s="4">
+        <v>11</v>
+      </c>
+      <c r="C192" s="4">
+        <v>5</v>
+      </c>
+      <c r="D192" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A193" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B193" s="4">
+        <v>12</v>
+      </c>
+      <c r="C193" s="4">
+        <v>5</v>
+      </c>
+      <c r="D193" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A194" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B194" s="4">
+        <v>1</v>
+      </c>
+      <c r="C194" s="4">
+        <v>5</v>
+      </c>
+      <c r="D194" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A195" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B195" s="4">
+        <v>2</v>
+      </c>
+      <c r="C195" s="4">
+        <v>5</v>
+      </c>
+      <c r="D195" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A196" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B196" s="4">
+        <v>3</v>
+      </c>
+      <c r="C196" s="4">
+        <v>5</v>
+      </c>
+      <c r="D196" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A197" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B197" s="4">
+        <v>4</v>
+      </c>
+      <c r="C197" s="4">
+        <v>5</v>
+      </c>
+      <c r="D197" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A198" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B198" s="4">
+        <v>5</v>
+      </c>
+      <c r="C198" s="4">
+        <v>5</v>
+      </c>
+      <c r="D198" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A199" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B199" s="4">
+        <v>6</v>
+      </c>
+      <c r="C199" s="4">
+        <v>5</v>
+      </c>
+      <c r="D199" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A200" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B200" s="4">
+        <v>7</v>
+      </c>
+      <c r="C200" s="4">
+        <v>5</v>
+      </c>
+      <c r="D200" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A201" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B201" s="4">
+        <v>8</v>
+      </c>
+      <c r="C201" s="4">
+        <v>5</v>
+      </c>
+      <c r="D201" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A202" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B202" s="4">
+        <v>9</v>
+      </c>
+      <c r="C202" s="4">
+        <v>5</v>
+      </c>
+      <c r="D202" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A203" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B203" s="4">
+        <v>10</v>
+      </c>
+      <c r="C203" s="4">
+        <v>5</v>
+      </c>
+      <c r="D203" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A204" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B204" s="4">
+        <v>11</v>
+      </c>
+      <c r="C204" s="4">
+        <v>5</v>
+      </c>
+      <c r="D204" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A205" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B205" s="4">
+        <v>12</v>
+      </c>
+      <c r="C205" s="4">
+        <v>5</v>
+      </c>
+      <c r="D205" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A206" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B206" s="4">
+        <v>1</v>
+      </c>
+      <c r="C206" s="4">
+        <v>5</v>
+      </c>
+      <c r="D206" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A207" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B207" s="4">
+        <v>2</v>
+      </c>
+      <c r="C207" s="4">
+        <v>5</v>
+      </c>
+      <c r="D207" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A208" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B208" s="4">
+        <v>3</v>
+      </c>
+      <c r="C208" s="4">
+        <v>5</v>
+      </c>
+      <c r="D208" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A209" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B209" s="4">
+        <v>4</v>
+      </c>
+      <c r="C209" s="4">
+        <v>5</v>
+      </c>
+      <c r="D209" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A210" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B210" s="4">
+        <v>5</v>
+      </c>
+      <c r="C210" s="4">
+        <v>5</v>
+      </c>
+      <c r="D210" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A211" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B211" s="4">
+        <v>6</v>
+      </c>
+      <c r="C211" s="4">
+        <v>5</v>
+      </c>
+      <c r="D211" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A212" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B212" s="4">
+        <v>7</v>
+      </c>
+      <c r="C212" s="4">
+        <v>5</v>
+      </c>
+      <c r="D212" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A213" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B213" s="4">
+        <v>8</v>
+      </c>
+      <c r="C213" s="4">
+        <v>5</v>
+      </c>
+      <c r="D213" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A214" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B214" s="4">
+        <v>9</v>
+      </c>
+      <c r="C214" s="4">
+        <v>5</v>
+      </c>
+      <c r="D214" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A215" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B215" s="4">
+        <v>10</v>
+      </c>
+      <c r="C215" s="4">
+        <v>5</v>
+      </c>
+      <c r="D215" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A216" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B216" s="4">
+        <v>11</v>
+      </c>
+      <c r="C216" s="4">
+        <v>5</v>
+      </c>
+      <c r="D216" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A217" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B217" s="4">
+        <v>12</v>
+      </c>
+      <c r="C217" s="4">
+        <v>5</v>
+      </c>
+      <c r="D217" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A218" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B218" s="4">
+        <v>1</v>
+      </c>
+      <c r="C218" s="4">
+        <v>5</v>
+      </c>
+      <c r="D218" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A219" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B219" s="4">
+        <v>2</v>
+      </c>
+      <c r="C219" s="4">
+        <v>5</v>
+      </c>
+      <c r="D219" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A220" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B220" s="4">
+        <v>3</v>
+      </c>
+      <c r="C220" s="4">
+        <v>5</v>
+      </c>
+      <c r="D220" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A221" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B221" s="4">
+        <v>4</v>
+      </c>
+      <c r="C221" s="4">
+        <v>5</v>
+      </c>
+      <c r="D221" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A222" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B222" s="4">
+        <v>5</v>
+      </c>
+      <c r="C222" s="4">
+        <v>5</v>
+      </c>
+      <c r="D222" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A223" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B223" s="4">
+        <v>6</v>
+      </c>
+      <c r="C223" s="4">
+        <v>5</v>
+      </c>
+      <c r="D223" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A224" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B224" s="4">
+        <v>7</v>
+      </c>
+      <c r="C224" s="4">
+        <v>5</v>
+      </c>
+      <c r="D224" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A225" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B225" s="4">
+        <v>8</v>
+      </c>
+      <c r="C225" s="4">
+        <v>5</v>
+      </c>
+      <c r="D225" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A226" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B226" s="4">
+        <v>9</v>
+      </c>
+      <c r="C226" s="4">
+        <v>5</v>
+      </c>
+      <c r="D226" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A227" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B227" s="4">
+        <v>10</v>
+      </c>
+      <c r="C227" s="4">
+        <v>5</v>
+      </c>
+      <c r="D227" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A228" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B228" s="4">
+        <v>11</v>
+      </c>
+      <c r="C228" s="4">
+        <v>5</v>
+      </c>
+      <c r="D228" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A229" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B229" s="4">
+        <v>12</v>
+      </c>
+      <c r="C229" s="4">
+        <v>5</v>
+      </c>
+      <c r="D229" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A230" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B230" s="4">
+        <v>1</v>
+      </c>
+      <c r="C230" s="4">
+        <v>5</v>
+      </c>
+      <c r="D230" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A231" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B231" s="4">
+        <v>2</v>
+      </c>
+      <c r="C231" s="4">
+        <v>5</v>
+      </c>
+      <c r="D231" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A232" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B232" s="4">
+        <v>3</v>
+      </c>
+      <c r="C232" s="4">
+        <v>5</v>
+      </c>
+      <c r="D232" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A233" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B233" s="4">
+        <v>4</v>
+      </c>
+      <c r="C233" s="4">
+        <v>5</v>
+      </c>
+      <c r="D233" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A234" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B234" s="4">
+        <v>5</v>
+      </c>
+      <c r="C234" s="4">
+        <v>5</v>
+      </c>
+      <c r="D234" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A235" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B235" s="4">
+        <v>6</v>
+      </c>
+      <c r="C235" s="4">
+        <v>5</v>
+      </c>
+      <c r="D235" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A236" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B236" s="4">
+        <v>7</v>
+      </c>
+      <c r="C236" s="4">
+        <v>5</v>
+      </c>
+      <c r="D236" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A237" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B237" s="4">
+        <v>8</v>
+      </c>
+      <c r="C237" s="4">
+        <v>5</v>
+      </c>
+      <c r="D237" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A238" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B238" s="4">
+        <v>9</v>
+      </c>
+      <c r="C238" s="4">
+        <v>5</v>
+      </c>
+      <c r="D238" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A239" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B239" s="4">
+        <v>10</v>
+      </c>
+      <c r="C239" s="4">
+        <v>5</v>
+      </c>
+      <c r="D239" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="240" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A240" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B240" s="4">
+        <v>11</v>
+      </c>
+      <c r="C240" s="4">
+        <v>5</v>
+      </c>
+      <c r="D240" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A241" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B241" s="4">
+        <v>12</v>
+      </c>
+      <c r="C241" s="4">
+        <v>5</v>
+      </c>
+      <c r="D241" s="4">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
GR and PCM under the infl of sedi are working - hooray! Next steps: add SS impacts on fert
</commit_message>
<xml_diff>
--- a/coral_data_and_custom_parameters.xlsx
+++ b/coral_data_and_custom_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uq-my.sharepoint.com/personal/uqrbutto_uq_edu_au/Documents/PhD_proj_pollution_on_coral_reefs/Coral-Model-Rio_sediment_extension/Coral-Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32B717CB-20CE-4090-85C7-148C11B2FA28}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53B47F0D-9345-4EC6-8BE8-481337A47E52}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-4290" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-4290" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Real_Cover" sheetId="1" r:id="rId1"/>
@@ -219,6 +219,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1948,10 +1952,10 @@
         <v>1</v>
       </c>
       <c r="C14" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D14" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -1962,10 +1966,10 @@
         <v>2</v>
       </c>
       <c r="C15" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D15" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
@@ -1976,10 +1980,10 @@
         <v>3</v>
       </c>
       <c r="C16" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D16" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
@@ -1990,10 +1994,10 @@
         <v>4</v>
       </c>
       <c r="C17" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D17" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -2004,10 +2008,10 @@
         <v>5</v>
       </c>
       <c r="C18" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D18" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -2018,10 +2022,10 @@
         <v>6</v>
       </c>
       <c r="C19" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D19" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -2032,10 +2036,10 @@
         <v>7</v>
       </c>
       <c r="C20" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D20" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -2046,10 +2050,10 @@
         <v>8</v>
       </c>
       <c r="C21" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D21" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -2060,10 +2064,10 @@
         <v>9</v>
       </c>
       <c r="C22" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D22" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -2074,10 +2078,10 @@
         <v>10</v>
       </c>
       <c r="C23" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D23" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -2088,10 +2092,10 @@
         <v>11</v>
       </c>
       <c r="C24" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D24" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -2102,10 +2106,10 @@
         <v>12</v>
       </c>
       <c r="C25" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D25" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -2623,7 +2627,7 @@
         <v>5</v>
       </c>
       <c r="D62" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
@@ -2637,7 +2641,7 @@
         <v>5</v>
       </c>
       <c r="D63" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
@@ -2651,7 +2655,7 @@
         <v>5</v>
       </c>
       <c r="D64" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
@@ -2665,7 +2669,7 @@
         <v>5</v>
       </c>
       <c r="D65" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
@@ -2679,7 +2683,7 @@
         <v>5</v>
       </c>
       <c r="D66" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
@@ -2693,7 +2697,7 @@
         <v>5</v>
       </c>
       <c r="D67" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
@@ -2707,7 +2711,7 @@
         <v>5</v>
       </c>
       <c r="D68" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
@@ -2721,7 +2725,7 @@
         <v>5</v>
       </c>
       <c r="D69" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
@@ -2735,7 +2739,7 @@
         <v>5</v>
       </c>
       <c r="D70" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
@@ -2749,7 +2753,7 @@
         <v>5</v>
       </c>
       <c r="D71" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
@@ -2763,7 +2767,7 @@
         <v>5</v>
       </c>
       <c r="D72" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
@@ -2777,7 +2781,7 @@
         <v>5</v>
       </c>
       <c r="D73" s="4">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
removed some fallbacks that might conceal errors. current issue: rerunning the model script produces different outcomes. liky cause: random state set for script not independently for each model run
</commit_message>
<xml_diff>
--- a/coral_data_and_custom_parameters.xlsx
+++ b/coral_data_and_custom_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uq-my.sharepoint.com/personal/uqrbutto_uq_edu_au/Documents/PhD_proj_pollution_on_coral_reefs/Coral-Model-Rio_sediment_extension/Coral-Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53B47F0D-9345-4EC6-8BE8-481337A47E52}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CB8C13A-868F-44F3-8DDF-31542D3C845C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-4290" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -219,10 +219,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1761,6 +1757,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E132077E-EAF7-4017-9CD9-9B94D708D64A}">
   <dimension ref="A1:D241"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="27" customWidth="1"/>
+    <col min="4" max="4" width="30.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
@@ -2627,7 +2627,7 @@
         <v>5</v>
       </c>
       <c r="D62" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
@@ -2641,7 +2641,7 @@
         <v>5</v>
       </c>
       <c r="D63" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
@@ -2655,7 +2655,7 @@
         <v>5</v>
       </c>
       <c r="D64" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
@@ -2669,7 +2669,7 @@
         <v>5</v>
       </c>
       <c r="D65" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
@@ -2683,7 +2683,7 @@
         <v>5</v>
       </c>
       <c r="D66" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
@@ -2697,7 +2697,7 @@
         <v>5</v>
       </c>
       <c r="D67" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
@@ -2711,7 +2711,7 @@
         <v>5</v>
       </c>
       <c r="D68" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
@@ -2725,7 +2725,7 @@
         <v>5</v>
       </c>
       <c r="D69" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
@@ -2739,7 +2739,7 @@
         <v>5</v>
       </c>
       <c r="D70" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
@@ -2753,7 +2753,7 @@
         <v>5</v>
       </c>
       <c r="D71" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
@@ -2767,7 +2767,7 @@
         <v>5</v>
       </c>
       <c r="D72" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
@@ -2781,7 +2781,7 @@
         <v>5</v>
       </c>
       <c r="D73" s="4">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
PCM additive. runs everything i sowkring. NEXT: make impacts of sedi, cyclne, bleaching, additive.
</commit_message>
<xml_diff>
--- a/coral_data_and_custom_parameters.xlsx
+++ b/coral_data_and_custom_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uq-my.sharepoint.com/personal/uqrbutto_uq_edu_au/Documents/PhD_proj_pollution_on_coral_reefs/Coral-Model-Rio_sediment_extension/Coral-Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="132" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CB8C13A-868F-44F3-8DDF-31542D3C845C}"/>
+  <xr:revisionPtr revIDLastSave="203" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7432A9EC-28D2-4B59-997E-3AE561FE1C21}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-4290" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1784,10 +1784,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D2" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1798,10 +1798,10 @@
         <v>2</v>
       </c>
       <c r="C3" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D3" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1812,10 +1812,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D4" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -1826,10 +1826,10 @@
         <v>4</v>
       </c>
       <c r="C5" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D5" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -1840,10 +1840,10 @@
         <v>5</v>
       </c>
       <c r="C6" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D6" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -1854,10 +1854,10 @@
         <v>6</v>
       </c>
       <c r="C7" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D7" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -1868,10 +1868,10 @@
         <v>7</v>
       </c>
       <c r="C8" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D8" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -1882,10 +1882,10 @@
         <v>8</v>
       </c>
       <c r="C9" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D9" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -1896,10 +1896,10 @@
         <v>9</v>
       </c>
       <c r="C10" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D10" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -1910,10 +1910,10 @@
         <v>10</v>
       </c>
       <c r="C11" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D11" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -1924,10 +1924,10 @@
         <v>11</v>
       </c>
       <c r="C12" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D12" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -1938,10 +1938,10 @@
         <v>12</v>
       </c>
       <c r="C13" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D13" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -1952,10 +1952,10 @@
         <v>1</v>
       </c>
       <c r="C14" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D14" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -1966,10 +1966,10 @@
         <v>2</v>
       </c>
       <c r="C15" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D15" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
@@ -1980,10 +1980,10 @@
         <v>3</v>
       </c>
       <c r="C16" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D16" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
@@ -1994,10 +1994,10 @@
         <v>4</v>
       </c>
       <c r="C17" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D17" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -2008,10 +2008,10 @@
         <v>5</v>
       </c>
       <c r="C18" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D18" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -2022,10 +2022,10 @@
         <v>6</v>
       </c>
       <c r="C19" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D19" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -2036,10 +2036,10 @@
         <v>7</v>
       </c>
       <c r="C20" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D20" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -2050,10 +2050,10 @@
         <v>8</v>
       </c>
       <c r="C21" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D21" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -2064,10 +2064,10 @@
         <v>9</v>
       </c>
       <c r="C22" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D22" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -2078,10 +2078,10 @@
         <v>10</v>
       </c>
       <c r="C23" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D23" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -2092,10 +2092,10 @@
         <v>11</v>
       </c>
       <c r="C24" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D24" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -2106,10 +2106,10 @@
         <v>12</v>
       </c>
       <c r="C25" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D25" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -2120,10 +2120,10 @@
         <v>1</v>
       </c>
       <c r="C26" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D26" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -2134,10 +2134,10 @@
         <v>2</v>
       </c>
       <c r="C27" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D27" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
@@ -2148,10 +2148,10 @@
         <v>3</v>
       </c>
       <c r="C28" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D28" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -2162,10 +2162,10 @@
         <v>4</v>
       </c>
       <c r="C29" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D29" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
@@ -2176,10 +2176,10 @@
         <v>5</v>
       </c>
       <c r="C30" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D30" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
@@ -2190,10 +2190,10 @@
         <v>6</v>
       </c>
       <c r="C31" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D31" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
@@ -2204,10 +2204,10 @@
         <v>7</v>
       </c>
       <c r="C32" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D32" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -2218,10 +2218,10 @@
         <v>8</v>
       </c>
       <c r="C33" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D33" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
@@ -2232,10 +2232,10 @@
         <v>9</v>
       </c>
       <c r="C34" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D34" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -2246,10 +2246,10 @@
         <v>10</v>
       </c>
       <c r="C35" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D35" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -2260,10 +2260,10 @@
         <v>11</v>
       </c>
       <c r="C36" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D36" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
@@ -2274,10 +2274,10 @@
         <v>12</v>
       </c>
       <c r="C37" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D37" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -2288,10 +2288,10 @@
         <v>1</v>
       </c>
       <c r="C38" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D38" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -2302,10 +2302,10 @@
         <v>2</v>
       </c>
       <c r="C39" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D39" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
@@ -2316,10 +2316,10 @@
         <v>3</v>
       </c>
       <c r="C40" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D40" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
@@ -2330,10 +2330,10 @@
         <v>4</v>
       </c>
       <c r="C41" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D41" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
@@ -2344,10 +2344,10 @@
         <v>5</v>
       </c>
       <c r="C42" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D42" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -2358,10 +2358,10 @@
         <v>6</v>
       </c>
       <c r="C43" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D43" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
@@ -2372,10 +2372,10 @@
         <v>7</v>
       </c>
       <c r="C44" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D44" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
@@ -2386,10 +2386,10 @@
         <v>8</v>
       </c>
       <c r="C45" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D45" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
@@ -2400,10 +2400,10 @@
         <v>9</v>
       </c>
       <c r="C46" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D46" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
@@ -2414,10 +2414,10 @@
         <v>10</v>
       </c>
       <c r="C47" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D47" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
@@ -2428,10 +2428,10 @@
         <v>11</v>
       </c>
       <c r="C48" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D48" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
@@ -2442,10 +2442,10 @@
         <v>12</v>
       </c>
       <c r="C49" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D49" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
@@ -2456,10 +2456,10 @@
         <v>1</v>
       </c>
       <c r="C50" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D50" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
@@ -2470,10 +2470,10 @@
         <v>2</v>
       </c>
       <c r="C51" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D51" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
@@ -2484,10 +2484,10 @@
         <v>3</v>
       </c>
       <c r="C52" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D52" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
@@ -2498,10 +2498,10 @@
         <v>4</v>
       </c>
       <c r="C53" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D53" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
@@ -2512,10 +2512,10 @@
         <v>5</v>
       </c>
       <c r="C54" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D54" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
@@ -2526,10 +2526,10 @@
         <v>6</v>
       </c>
       <c r="C55" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D55" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
@@ -2540,10 +2540,10 @@
         <v>7</v>
       </c>
       <c r="C56" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D56" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
@@ -2554,10 +2554,10 @@
         <v>8</v>
       </c>
       <c r="C57" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D57" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
@@ -2568,10 +2568,10 @@
         <v>9</v>
       </c>
       <c r="C58" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D58" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
@@ -2582,10 +2582,10 @@
         <v>10</v>
       </c>
       <c r="C59" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D59" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
@@ -2596,10 +2596,10 @@
         <v>11</v>
       </c>
       <c r="C60" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D60" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
@@ -2610,10 +2610,10 @@
         <v>12</v>
       </c>
       <c r="C61" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D61" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
@@ -2624,10 +2624,10 @@
         <v>1</v>
       </c>
       <c r="C62" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D62" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
@@ -2638,10 +2638,10 @@
         <v>2</v>
       </c>
       <c r="C63" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D63" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
@@ -2652,10 +2652,10 @@
         <v>3</v>
       </c>
       <c r="C64" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D64" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
@@ -2666,10 +2666,10 @@
         <v>4</v>
       </c>
       <c r="C65" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D65" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
@@ -2680,10 +2680,10 @@
         <v>5</v>
       </c>
       <c r="C66" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D66" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
@@ -2694,10 +2694,10 @@
         <v>6</v>
       </c>
       <c r="C67" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D67" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
@@ -2708,10 +2708,10 @@
         <v>7</v>
       </c>
       <c r="C68" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D68" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
@@ -2722,10 +2722,10 @@
         <v>8</v>
       </c>
       <c r="C69" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D69" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
@@ -2736,10 +2736,10 @@
         <v>9</v>
       </c>
       <c r="C70" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D70" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
@@ -2750,10 +2750,10 @@
         <v>10</v>
       </c>
       <c r="C71" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D71" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
@@ -2764,10 +2764,10 @@
         <v>11</v>
       </c>
       <c r="C72" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D72" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
@@ -2778,10 +2778,10 @@
         <v>12</v>
       </c>
       <c r="C73" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D73" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
@@ -2792,10 +2792,10 @@
         <v>1</v>
       </c>
       <c r="C74" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D74" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
@@ -2806,10 +2806,10 @@
         <v>2</v>
       </c>
       <c r="C75" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D75" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
@@ -2820,10 +2820,10 @@
         <v>3</v>
       </c>
       <c r="C76" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D76" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
@@ -2834,10 +2834,10 @@
         <v>4</v>
       </c>
       <c r="C77" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D77" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
@@ -2848,10 +2848,10 @@
         <v>5</v>
       </c>
       <c r="C78" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D78" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
@@ -2862,10 +2862,10 @@
         <v>6</v>
       </c>
       <c r="C79" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D79" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
@@ -2876,10 +2876,10 @@
         <v>7</v>
       </c>
       <c r="C80" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D80" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
@@ -2890,10 +2890,10 @@
         <v>8</v>
       </c>
       <c r="C81" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D81" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
@@ -2904,10 +2904,10 @@
         <v>9</v>
       </c>
       <c r="C82" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D82" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
@@ -2918,10 +2918,10 @@
         <v>10</v>
       </c>
       <c r="C83" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D83" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
@@ -2932,10 +2932,10 @@
         <v>11</v>
       </c>
       <c r="C84" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D84" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
@@ -2946,10 +2946,10 @@
         <v>12</v>
       </c>
       <c r="C85" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D85" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
@@ -2960,10 +2960,10 @@
         <v>1</v>
       </c>
       <c r="C86" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D86" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
@@ -2974,10 +2974,10 @@
         <v>2</v>
       </c>
       <c r="C87" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D87" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
@@ -2988,10 +2988,10 @@
         <v>3</v>
       </c>
       <c r="C88" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D88" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
@@ -3002,10 +3002,10 @@
         <v>4</v>
       </c>
       <c r="C89" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D89" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
@@ -3016,10 +3016,10 @@
         <v>5</v>
       </c>
       <c r="C90" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D90" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
@@ -3030,10 +3030,10 @@
         <v>6</v>
       </c>
       <c r="C91" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D91" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
@@ -3044,10 +3044,10 @@
         <v>7</v>
       </c>
       <c r="C92" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D92" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.35">
@@ -3058,10 +3058,10 @@
         <v>8</v>
       </c>
       <c r="C93" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D93" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.35">
@@ -3072,10 +3072,10 @@
         <v>9</v>
       </c>
       <c r="C94" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D94" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
@@ -3086,10 +3086,10 @@
         <v>10</v>
       </c>
       <c r="C95" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D95" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
@@ -3100,10 +3100,10 @@
         <v>11</v>
       </c>
       <c r="C96" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D96" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
@@ -3114,10 +3114,10 @@
         <v>12</v>
       </c>
       <c r="C97" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D97" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.35">
@@ -3128,10 +3128,10 @@
         <v>1</v>
       </c>
       <c r="C98" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D98" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
@@ -3142,10 +3142,10 @@
         <v>2</v>
       </c>
       <c r="C99" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D99" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.35">
@@ -3156,10 +3156,10 @@
         <v>3</v>
       </c>
       <c r="C100" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D100" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.35">
@@ -3170,10 +3170,10 @@
         <v>4</v>
       </c>
       <c r="C101" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D101" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.35">
@@ -3184,10 +3184,10 @@
         <v>5</v>
       </c>
       <c r="C102" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D102" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.35">
@@ -3198,10 +3198,10 @@
         <v>6</v>
       </c>
       <c r="C103" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D103" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.35">
@@ -3212,10 +3212,10 @@
         <v>7</v>
       </c>
       <c r="C104" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D104" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.35">
@@ -3226,10 +3226,10 @@
         <v>8</v>
       </c>
       <c r="C105" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D105" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
@@ -3240,10 +3240,10 @@
         <v>9</v>
       </c>
       <c r="C106" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D106" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.35">
@@ -3254,10 +3254,10 @@
         <v>10</v>
       </c>
       <c r="C107" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D107" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.35">
@@ -3268,10 +3268,10 @@
         <v>11</v>
       </c>
       <c r="C108" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D108" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.35">
@@ -3282,10 +3282,10 @@
         <v>12</v>
       </c>
       <c r="C109" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D109" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.35">
@@ -3296,10 +3296,10 @@
         <v>1</v>
       </c>
       <c r="C110" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D110" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.35">
@@ -3310,10 +3310,10 @@
         <v>2</v>
       </c>
       <c r="C111" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D111" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.35">
@@ -3324,10 +3324,10 @@
         <v>3</v>
       </c>
       <c r="C112" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D112" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.35">
@@ -3338,10 +3338,10 @@
         <v>4</v>
       </c>
       <c r="C113" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D113" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.35">
@@ -3352,10 +3352,10 @@
         <v>5</v>
       </c>
       <c r="C114" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D114" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.35">
@@ -3366,10 +3366,10 @@
         <v>6</v>
       </c>
       <c r="C115" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D115" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.35">
@@ -3380,10 +3380,10 @@
         <v>7</v>
       </c>
       <c r="C116" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D116" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.35">
@@ -3394,10 +3394,10 @@
         <v>8</v>
       </c>
       <c r="C117" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D117" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.35">
@@ -3408,10 +3408,10 @@
         <v>9</v>
       </c>
       <c r="C118" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D118" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.35">
@@ -3422,10 +3422,10 @@
         <v>10</v>
       </c>
       <c r="C119" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D119" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.35">
@@ -3436,10 +3436,10 @@
         <v>11</v>
       </c>
       <c r="C120" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D120" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.35">
@@ -3450,10 +3450,10 @@
         <v>12</v>
       </c>
       <c r="C121" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D121" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.35">
@@ -3464,10 +3464,10 @@
         <v>1</v>
       </c>
       <c r="C122" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D122" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.35">
@@ -3478,10 +3478,10 @@
         <v>2</v>
       </c>
       <c r="C123" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D123" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.35">
@@ -3492,10 +3492,10 @@
         <v>3</v>
       </c>
       <c r="C124" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D124" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.35">
@@ -3506,10 +3506,10 @@
         <v>4</v>
       </c>
       <c r="C125" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D125" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.35">
@@ -3520,10 +3520,10 @@
         <v>5</v>
       </c>
       <c r="C126" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D126" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.35">
@@ -3534,10 +3534,10 @@
         <v>6</v>
       </c>
       <c r="C127" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D127" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.35">
@@ -3548,10 +3548,10 @@
         <v>7</v>
       </c>
       <c r="C128" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D128" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.35">
@@ -3562,10 +3562,10 @@
         <v>8</v>
       </c>
       <c r="C129" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D129" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.35">
@@ -3576,10 +3576,10 @@
         <v>9</v>
       </c>
       <c r="C130" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D130" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.35">
@@ -3590,10 +3590,10 @@
         <v>10</v>
       </c>
       <c r="C131" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D131" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.35">
@@ -3604,10 +3604,10 @@
         <v>11</v>
       </c>
       <c r="C132" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D132" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.35">
@@ -3618,10 +3618,10 @@
         <v>12</v>
       </c>
       <c r="C133" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D133" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.35">
@@ -3632,10 +3632,10 @@
         <v>1</v>
       </c>
       <c r="C134" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D134" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.35">
@@ -3646,10 +3646,10 @@
         <v>2</v>
       </c>
       <c r="C135" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D135" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.35">
@@ -3660,10 +3660,10 @@
         <v>3</v>
       </c>
       <c r="C136" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D136" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.35">
@@ -3674,10 +3674,10 @@
         <v>4</v>
       </c>
       <c r="C137" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D137" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.35">
@@ -3688,10 +3688,10 @@
         <v>5</v>
       </c>
       <c r="C138" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D138" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.35">
@@ -3702,10 +3702,10 @@
         <v>6</v>
       </c>
       <c r="C139" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D139" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.35">
@@ -3716,10 +3716,10 @@
         <v>7</v>
       </c>
       <c r="C140" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D140" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.35">
@@ -3730,10 +3730,10 @@
         <v>8</v>
       </c>
       <c r="C141" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D141" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.35">
@@ -3744,10 +3744,10 @@
         <v>9</v>
       </c>
       <c r="C142" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D142" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.35">
@@ -3758,10 +3758,10 @@
         <v>10</v>
       </c>
       <c r="C143" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D143" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.35">
@@ -3772,10 +3772,10 @@
         <v>11</v>
       </c>
       <c r="C144" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D144" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.35">
@@ -3786,10 +3786,10 @@
         <v>12</v>
       </c>
       <c r="C145" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D145" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.35">
@@ -3800,10 +3800,10 @@
         <v>1</v>
       </c>
       <c r="C146" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D146" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.35">
@@ -3814,10 +3814,10 @@
         <v>2</v>
       </c>
       <c r="C147" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D147" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.35">
@@ -3828,10 +3828,10 @@
         <v>3</v>
       </c>
       <c r="C148" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D148" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.35">
@@ -3842,10 +3842,10 @@
         <v>4</v>
       </c>
       <c r="C149" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D149" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.35">
@@ -3856,10 +3856,10 @@
         <v>5</v>
       </c>
       <c r="C150" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D150" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.35">
@@ -3870,10 +3870,10 @@
         <v>6</v>
       </c>
       <c r="C151" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D151" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.35">
@@ -3884,10 +3884,10 @@
         <v>7</v>
       </c>
       <c r="C152" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D152" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.35">
@@ -3898,10 +3898,10 @@
         <v>8</v>
       </c>
       <c r="C153" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D153" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.35">
@@ -3912,10 +3912,10 @@
         <v>9</v>
       </c>
       <c r="C154" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D154" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.35">
@@ -3926,10 +3926,10 @@
         <v>10</v>
       </c>
       <c r="C155" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D155" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.35">
@@ -3940,10 +3940,10 @@
         <v>11</v>
       </c>
       <c r="C156" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D156" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.35">
@@ -3954,10 +3954,10 @@
         <v>12</v>
       </c>
       <c r="C157" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D157" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.35">
@@ -3968,10 +3968,10 @@
         <v>1</v>
       </c>
       <c r="C158" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D158" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.35">
@@ -3982,10 +3982,10 @@
         <v>2</v>
       </c>
       <c r="C159" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D159" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.35">
@@ -3996,10 +3996,10 @@
         <v>3</v>
       </c>
       <c r="C160" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D160" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.35">
@@ -4010,10 +4010,10 @@
         <v>4</v>
       </c>
       <c r="C161" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D161" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.35">
@@ -4024,10 +4024,10 @@
         <v>5</v>
       </c>
       <c r="C162" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D162" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.35">
@@ -4038,10 +4038,10 @@
         <v>6</v>
       </c>
       <c r="C163" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D163" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.35">
@@ -4052,10 +4052,10 @@
         <v>7</v>
       </c>
       <c r="C164" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D164" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.35">
@@ -4066,10 +4066,10 @@
         <v>8</v>
       </c>
       <c r="C165" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D165" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.35">
@@ -4080,10 +4080,10 @@
         <v>9</v>
       </c>
       <c r="C166" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D166" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.35">
@@ -4094,10 +4094,10 @@
         <v>10</v>
       </c>
       <c r="C167" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D167" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.35">
@@ -4108,10 +4108,10 @@
         <v>11</v>
       </c>
       <c r="C168" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D168" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.35">
@@ -4122,10 +4122,10 @@
         <v>12</v>
       </c>
       <c r="C169" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D169" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.35">
@@ -4136,10 +4136,10 @@
         <v>1</v>
       </c>
       <c r="C170" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D170" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.35">
@@ -4150,10 +4150,10 @@
         <v>2</v>
       </c>
       <c r="C171" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D171" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.35">
@@ -4164,10 +4164,10 @@
         <v>3</v>
       </c>
       <c r="C172" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D172" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.35">
@@ -4178,10 +4178,10 @@
         <v>4</v>
       </c>
       <c r="C173" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D173" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.35">
@@ -4192,10 +4192,10 @@
         <v>5</v>
       </c>
       <c r="C174" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D174" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.35">
@@ -4206,10 +4206,10 @@
         <v>6</v>
       </c>
       <c r="C175" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D175" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.35">
@@ -4220,10 +4220,10 @@
         <v>7</v>
       </c>
       <c r="C176" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D176" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.35">
@@ -4234,10 +4234,10 @@
         <v>8</v>
       </c>
       <c r="C177" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D177" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.35">
@@ -4248,10 +4248,10 @@
         <v>9</v>
       </c>
       <c r="C178" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D178" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.35">
@@ -4262,10 +4262,10 @@
         <v>10</v>
       </c>
       <c r="C179" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D179" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.35">
@@ -4276,10 +4276,10 @@
         <v>11</v>
       </c>
       <c r="C180" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D180" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.35">
@@ -4290,10 +4290,10 @@
         <v>12</v>
       </c>
       <c r="C181" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D181" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.35">
@@ -4304,10 +4304,10 @@
         <v>1</v>
       </c>
       <c r="C182" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D182" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.35">
@@ -4318,10 +4318,10 @@
         <v>2</v>
       </c>
       <c r="C183" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D183" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.35">
@@ -4332,10 +4332,10 @@
         <v>3</v>
       </c>
       <c r="C184" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D184" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.35">
@@ -4346,10 +4346,10 @@
         <v>4</v>
       </c>
       <c r="C185" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D185" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.35">
@@ -4360,10 +4360,10 @@
         <v>5</v>
       </c>
       <c r="C186" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D186" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.35">
@@ -4374,10 +4374,10 @@
         <v>6</v>
       </c>
       <c r="C187" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D187" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.35">
@@ -4388,10 +4388,10 @@
         <v>7</v>
       </c>
       <c r="C188" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D188" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.35">
@@ -4402,10 +4402,10 @@
         <v>8</v>
       </c>
       <c r="C189" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D189" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.35">
@@ -4416,10 +4416,10 @@
         <v>9</v>
       </c>
       <c r="C190" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D190" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.35">
@@ -4430,10 +4430,10 @@
         <v>10</v>
       </c>
       <c r="C191" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D191" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.35">
@@ -4444,10 +4444,10 @@
         <v>11</v>
       </c>
       <c r="C192" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D192" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.35">
@@ -4458,10 +4458,10 @@
         <v>12</v>
       </c>
       <c r="C193" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D193" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.35">
@@ -4472,10 +4472,10 @@
         <v>1</v>
       </c>
       <c r="C194" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D194" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.35">
@@ -4486,10 +4486,10 @@
         <v>2</v>
       </c>
       <c r="C195" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D195" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.35">
@@ -4500,10 +4500,10 @@
         <v>3</v>
       </c>
       <c r="C196" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D196" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.35">
@@ -4514,10 +4514,10 @@
         <v>4</v>
       </c>
       <c r="C197" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D197" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.35">
@@ -4528,10 +4528,10 @@
         <v>5</v>
       </c>
       <c r="C198" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D198" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.35">
@@ -4542,10 +4542,10 @@
         <v>6</v>
       </c>
       <c r="C199" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D199" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.35">
@@ -4556,10 +4556,10 @@
         <v>7</v>
       </c>
       <c r="C200" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D200" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.35">
@@ -4570,10 +4570,10 @@
         <v>8</v>
       </c>
       <c r="C201" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D201" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.35">
@@ -4584,10 +4584,10 @@
         <v>9</v>
       </c>
       <c r="C202" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D202" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.35">
@@ -4598,10 +4598,10 @@
         <v>10</v>
       </c>
       <c r="C203" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D203" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.35">
@@ -4612,10 +4612,10 @@
         <v>11</v>
       </c>
       <c r="C204" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D204" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.35">
@@ -4626,10 +4626,10 @@
         <v>12</v>
       </c>
       <c r="C205" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D205" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.35">
@@ -4640,10 +4640,10 @@
         <v>1</v>
       </c>
       <c r="C206" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D206" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.35">
@@ -4654,10 +4654,10 @@
         <v>2</v>
       </c>
       <c r="C207" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D207" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.35">
@@ -4668,10 +4668,10 @@
         <v>3</v>
       </c>
       <c r="C208" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D208" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.35">
@@ -4682,10 +4682,10 @@
         <v>4</v>
       </c>
       <c r="C209" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D209" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.35">
@@ -4696,10 +4696,10 @@
         <v>5</v>
       </c>
       <c r="C210" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D210" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.35">
@@ -4710,10 +4710,10 @@
         <v>6</v>
       </c>
       <c r="C211" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D211" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.35">
@@ -4724,10 +4724,10 @@
         <v>7</v>
       </c>
       <c r="C212" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D212" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.35">
@@ -4738,10 +4738,10 @@
         <v>8</v>
       </c>
       <c r="C213" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D213" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.35">
@@ -4752,10 +4752,10 @@
         <v>9</v>
       </c>
       <c r="C214" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D214" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.35">
@@ -4766,10 +4766,10 @@
         <v>10</v>
       </c>
       <c r="C215" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D215" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.35">
@@ -4780,10 +4780,10 @@
         <v>11</v>
       </c>
       <c r="C216" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D216" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.35">
@@ -4794,10 +4794,10 @@
         <v>12</v>
       </c>
       <c r="C217" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D217" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.35">
@@ -4808,10 +4808,10 @@
         <v>1</v>
       </c>
       <c r="C218" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D218" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.35">
@@ -4822,10 +4822,10 @@
         <v>2</v>
       </c>
       <c r="C219" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D219" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.35">
@@ -4836,10 +4836,10 @@
         <v>3</v>
       </c>
       <c r="C220" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D220" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.35">
@@ -4850,10 +4850,10 @@
         <v>4</v>
       </c>
       <c r="C221" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D221" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.35">
@@ -4864,10 +4864,10 @@
         <v>5</v>
       </c>
       <c r="C222" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D222" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.35">
@@ -4878,10 +4878,10 @@
         <v>6</v>
       </c>
       <c r="C223" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D223" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.35">
@@ -4892,10 +4892,10 @@
         <v>7</v>
       </c>
       <c r="C224" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D224" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.35">
@@ -4906,10 +4906,10 @@
         <v>8</v>
       </c>
       <c r="C225" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D225" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.35">
@@ -4920,10 +4920,10 @@
         <v>9</v>
       </c>
       <c r="C226" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D226" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.35">
@@ -4934,10 +4934,10 @@
         <v>10</v>
       </c>
       <c r="C227" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D227" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.35">
@@ -4948,10 +4948,10 @@
         <v>11</v>
       </c>
       <c r="C228" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D228" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.35">
@@ -4962,10 +4962,10 @@
         <v>12</v>
       </c>
       <c r="C229" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D229" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.35">
@@ -4976,10 +4976,10 @@
         <v>1</v>
       </c>
       <c r="C230" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D230" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.35">
@@ -4990,10 +4990,10 @@
         <v>2</v>
       </c>
       <c r="C231" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D231" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.35">
@@ -5004,10 +5004,10 @@
         <v>3</v>
       </c>
       <c r="C232" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D232" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.35">
@@ -5018,10 +5018,10 @@
         <v>4</v>
       </c>
       <c r="C233" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D233" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.35">
@@ -5032,10 +5032,10 @@
         <v>5</v>
       </c>
       <c r="C234" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D234" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.35">
@@ -5046,10 +5046,10 @@
         <v>6</v>
       </c>
       <c r="C235" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D235" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.35">
@@ -5060,10 +5060,10 @@
         <v>7</v>
       </c>
       <c r="C236" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D236" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.35">
@@ -5074,10 +5074,10 @@
         <v>8</v>
       </c>
       <c r="C237" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D237" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.35">
@@ -5088,10 +5088,10 @@
         <v>9</v>
       </c>
       <c r="C238" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D238" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.35">
@@ -5102,10 +5102,10 @@
         <v>10</v>
       </c>
       <c r="C239" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D239" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.35">
@@ -5116,10 +5116,10 @@
         <v>11</v>
       </c>
       <c r="C240" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D240" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.35">
@@ -5130,10 +5130,10 @@
         <v>12</v>
       </c>
       <c r="C241" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D241" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Saving changes before I extend the model to include default PSD based on regime, region, depth
</commit_message>
<xml_diff>
--- a/coral_data_and_custom_parameters.xlsx
+++ b/coral_data_and_custom_parameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uq-my.sharepoint.com/personal/uqrbutto_uq_edu_au/Documents/PhD_proj_pollution_on_coral_reefs/Coral-Model-Rio_sediment_extension/Coral-Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="203" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7432A9EC-28D2-4B59-997E-3AE561FE1C21}"/>
+  <xr:revisionPtr revIDLastSave="233" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4959E353-E602-4A0C-A2ED-8F991FFA353F}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-4290" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1636,7 +1636,7 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>2.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -1644,7 +1644,7 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1652,7 +1652,7 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -1784,10 +1784,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D2" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1798,10 +1798,10 @@
         <v>2</v>
       </c>
       <c r="C3" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D3" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1812,10 +1812,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D4" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -1826,10 +1826,10 @@
         <v>4</v>
       </c>
       <c r="C5" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D5" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -1840,10 +1840,10 @@
         <v>5</v>
       </c>
       <c r="C6" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D6" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -1854,10 +1854,10 @@
         <v>6</v>
       </c>
       <c r="C7" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D7" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -1868,10 +1868,10 @@
         <v>7</v>
       </c>
       <c r="C8" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D8" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -1882,10 +1882,10 @@
         <v>8</v>
       </c>
       <c r="C9" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D9" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -1896,10 +1896,10 @@
         <v>9</v>
       </c>
       <c r="C10" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D10" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -1910,10 +1910,10 @@
         <v>10</v>
       </c>
       <c r="C11" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D11" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -1924,10 +1924,10 @@
         <v>11</v>
       </c>
       <c r="C12" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D12" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -1938,10 +1938,10 @@
         <v>12</v>
       </c>
       <c r="C13" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D13" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -1952,10 +1952,10 @@
         <v>1</v>
       </c>
       <c r="C14" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D14" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -1966,10 +1966,10 @@
         <v>2</v>
       </c>
       <c r="C15" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D15" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
@@ -1980,10 +1980,10 @@
         <v>3</v>
       </c>
       <c r="C16" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D16" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
@@ -1994,10 +1994,10 @@
         <v>4</v>
       </c>
       <c r="C17" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D17" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -2008,10 +2008,10 @@
         <v>5</v>
       </c>
       <c r="C18" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D18" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -2022,10 +2022,10 @@
         <v>6</v>
       </c>
       <c r="C19" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D19" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -2036,10 +2036,10 @@
         <v>7</v>
       </c>
       <c r="C20" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D20" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -2050,10 +2050,10 @@
         <v>8</v>
       </c>
       <c r="C21" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D21" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -2064,10 +2064,10 @@
         <v>9</v>
       </c>
       <c r="C22" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D22" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -2078,10 +2078,10 @@
         <v>10</v>
       </c>
       <c r="C23" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D23" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -2092,10 +2092,10 @@
         <v>11</v>
       </c>
       <c r="C24" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D24" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -2106,10 +2106,10 @@
         <v>12</v>
       </c>
       <c r="C25" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D25" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -2120,10 +2120,10 @@
         <v>1</v>
       </c>
       <c r="C26" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D26" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -2134,10 +2134,10 @@
         <v>2</v>
       </c>
       <c r="C27" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D27" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
@@ -2148,10 +2148,10 @@
         <v>3</v>
       </c>
       <c r="C28" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D28" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -2162,10 +2162,10 @@
         <v>4</v>
       </c>
       <c r="C29" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D29" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
@@ -2176,10 +2176,10 @@
         <v>5</v>
       </c>
       <c r="C30" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D30" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
@@ -2190,10 +2190,10 @@
         <v>6</v>
       </c>
       <c r="C31" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D31" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
@@ -2204,10 +2204,10 @@
         <v>7</v>
       </c>
       <c r="C32" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D32" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -2218,10 +2218,10 @@
         <v>8</v>
       </c>
       <c r="C33" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D33" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
@@ -2232,10 +2232,10 @@
         <v>9</v>
       </c>
       <c r="C34" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D34" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -2246,10 +2246,10 @@
         <v>10</v>
       </c>
       <c r="C35" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D35" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -2260,10 +2260,10 @@
         <v>11</v>
       </c>
       <c r="C36" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D36" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
@@ -2274,10 +2274,10 @@
         <v>12</v>
       </c>
       <c r="C37" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D37" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -2288,10 +2288,10 @@
         <v>1</v>
       </c>
       <c r="C38" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D38" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -2302,10 +2302,10 @@
         <v>2</v>
       </c>
       <c r="C39" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D39" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
@@ -2316,10 +2316,10 @@
         <v>3</v>
       </c>
       <c r="C40" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D40" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
@@ -2330,10 +2330,10 @@
         <v>4</v>
       </c>
       <c r="C41" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D41" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
@@ -2344,10 +2344,10 @@
         <v>5</v>
       </c>
       <c r="C42" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D42" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -2358,10 +2358,10 @@
         <v>6</v>
       </c>
       <c r="C43" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D43" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
@@ -2372,10 +2372,10 @@
         <v>7</v>
       </c>
       <c r="C44" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D44" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
@@ -2386,10 +2386,10 @@
         <v>8</v>
       </c>
       <c r="C45" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D45" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
@@ -2400,10 +2400,10 @@
         <v>9</v>
       </c>
       <c r="C46" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D46" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
@@ -2414,10 +2414,10 @@
         <v>10</v>
       </c>
       <c r="C47" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D47" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
@@ -2428,10 +2428,10 @@
         <v>11</v>
       </c>
       <c r="C48" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D48" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
@@ -2442,10 +2442,10 @@
         <v>12</v>
       </c>
       <c r="C49" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D49" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
@@ -2456,10 +2456,10 @@
         <v>1</v>
       </c>
       <c r="C50" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D50" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
@@ -2470,10 +2470,10 @@
         <v>2</v>
       </c>
       <c r="C51" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D51" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
@@ -2484,10 +2484,10 @@
         <v>3</v>
       </c>
       <c r="C52" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D52" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
@@ -2498,10 +2498,10 @@
         <v>4</v>
       </c>
       <c r="C53" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D53" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
@@ -2512,10 +2512,10 @@
         <v>5</v>
       </c>
       <c r="C54" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D54" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
@@ -2526,10 +2526,10 @@
         <v>6</v>
       </c>
       <c r="C55" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D55" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
@@ -2540,10 +2540,10 @@
         <v>7</v>
       </c>
       <c r="C56" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D56" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
@@ -2554,10 +2554,10 @@
         <v>8</v>
       </c>
       <c r="C57" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D57" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
@@ -2568,10 +2568,10 @@
         <v>9</v>
       </c>
       <c r="C58" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D58" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
@@ -2582,10 +2582,10 @@
         <v>10</v>
       </c>
       <c r="C59" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D59" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
@@ -2596,10 +2596,10 @@
         <v>11</v>
       </c>
       <c r="C60" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D60" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
@@ -2610,10 +2610,10 @@
         <v>12</v>
       </c>
       <c r="C61" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D61" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
@@ -2624,10 +2624,10 @@
         <v>1</v>
       </c>
       <c r="C62" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D62" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
@@ -2638,10 +2638,10 @@
         <v>2</v>
       </c>
       <c r="C63" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D63" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
@@ -2652,10 +2652,10 @@
         <v>3</v>
       </c>
       <c r="C64" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D64" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
@@ -2666,10 +2666,10 @@
         <v>4</v>
       </c>
       <c r="C65" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D65" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
@@ -2680,10 +2680,10 @@
         <v>5</v>
       </c>
       <c r="C66" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D66" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
@@ -2694,10 +2694,10 @@
         <v>6</v>
       </c>
       <c r="C67" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D67" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
@@ -2708,10 +2708,10 @@
         <v>7</v>
       </c>
       <c r="C68" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D68" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
@@ -2722,10 +2722,10 @@
         <v>8</v>
       </c>
       <c r="C69" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D69" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
@@ -2736,10 +2736,10 @@
         <v>9</v>
       </c>
       <c r="C70" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D70" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
@@ -2750,10 +2750,10 @@
         <v>10</v>
       </c>
       <c r="C71" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D71" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
@@ -2764,10 +2764,10 @@
         <v>11</v>
       </c>
       <c r="C72" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D72" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
@@ -2778,10 +2778,10 @@
         <v>12</v>
       </c>
       <c r="C73" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D73" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
@@ -2792,10 +2792,10 @@
         <v>1</v>
       </c>
       <c r="C74" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D74" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
@@ -2806,10 +2806,10 @@
         <v>2</v>
       </c>
       <c r="C75" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D75" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
@@ -2820,10 +2820,10 @@
         <v>3</v>
       </c>
       <c r="C76" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D76" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
@@ -2834,10 +2834,10 @@
         <v>4</v>
       </c>
       <c r="C77" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D77" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
@@ -2848,10 +2848,10 @@
         <v>5</v>
       </c>
       <c r="C78" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D78" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
@@ -2862,10 +2862,10 @@
         <v>6</v>
       </c>
       <c r="C79" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D79" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
@@ -2876,10 +2876,10 @@
         <v>7</v>
       </c>
       <c r="C80" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D80" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
@@ -2890,10 +2890,10 @@
         <v>8</v>
       </c>
       <c r="C81" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D81" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
@@ -2904,10 +2904,10 @@
         <v>9</v>
       </c>
       <c r="C82" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D82" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
@@ -2918,10 +2918,10 @@
         <v>10</v>
       </c>
       <c r="C83" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D83" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
@@ -2932,10 +2932,10 @@
         <v>11</v>
       </c>
       <c r="C84" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D84" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
@@ -2946,10 +2946,10 @@
         <v>12</v>
       </c>
       <c r="C85" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D85" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
@@ -2960,10 +2960,10 @@
         <v>1</v>
       </c>
       <c r="C86" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D86" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
@@ -2974,10 +2974,10 @@
         <v>2</v>
       </c>
       <c r="C87" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D87" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
@@ -2988,10 +2988,10 @@
         <v>3</v>
       </c>
       <c r="C88" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D88" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
@@ -3002,10 +3002,10 @@
         <v>4</v>
       </c>
       <c r="C89" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D89" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
@@ -3016,10 +3016,10 @@
         <v>5</v>
       </c>
       <c r="C90" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D90" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
@@ -3030,10 +3030,10 @@
         <v>6</v>
       </c>
       <c r="C91" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D91" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
@@ -3044,10 +3044,10 @@
         <v>7</v>
       </c>
       <c r="C92" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D92" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.35">
@@ -3058,10 +3058,10 @@
         <v>8</v>
       </c>
       <c r="C93" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D93" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.35">
@@ -3072,10 +3072,10 @@
         <v>9</v>
       </c>
       <c r="C94" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D94" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
@@ -3086,10 +3086,10 @@
         <v>10</v>
       </c>
       <c r="C95" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D95" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
@@ -3100,10 +3100,10 @@
         <v>11</v>
       </c>
       <c r="C96" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D96" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
@@ -3114,10 +3114,10 @@
         <v>12</v>
       </c>
       <c r="C97" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D97" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.35">
@@ -3128,10 +3128,10 @@
         <v>1</v>
       </c>
       <c r="C98" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D98" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
@@ -3142,10 +3142,10 @@
         <v>2</v>
       </c>
       <c r="C99" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D99" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.35">
@@ -3156,10 +3156,10 @@
         <v>3</v>
       </c>
       <c r="C100" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D100" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.35">
@@ -3170,10 +3170,10 @@
         <v>4</v>
       </c>
       <c r="C101" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D101" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.35">
@@ -3184,10 +3184,10 @@
         <v>5</v>
       </c>
       <c r="C102" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D102" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.35">
@@ -3198,10 +3198,10 @@
         <v>6</v>
       </c>
       <c r="C103" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D103" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.35">
@@ -3212,10 +3212,10 @@
         <v>7</v>
       </c>
       <c r="C104" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D104" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.35">
@@ -3226,10 +3226,10 @@
         <v>8</v>
       </c>
       <c r="C105" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D105" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
@@ -3240,10 +3240,10 @@
         <v>9</v>
       </c>
       <c r="C106" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D106" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.35">
@@ -3254,10 +3254,10 @@
         <v>10</v>
       </c>
       <c r="C107" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D107" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.35">
@@ -3268,10 +3268,10 @@
         <v>11</v>
       </c>
       <c r="C108" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D108" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.35">
@@ -3282,10 +3282,10 @@
         <v>12</v>
       </c>
       <c r="C109" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D109" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.35">
@@ -3296,10 +3296,10 @@
         <v>1</v>
       </c>
       <c r="C110" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D110" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.35">
@@ -3310,10 +3310,10 @@
         <v>2</v>
       </c>
       <c r="C111" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D111" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.35">
@@ -3324,10 +3324,10 @@
         <v>3</v>
       </c>
       <c r="C112" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D112" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.35">
@@ -3338,10 +3338,10 @@
         <v>4</v>
       </c>
       <c r="C113" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D113" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.35">
@@ -3352,10 +3352,10 @@
         <v>5</v>
       </c>
       <c r="C114" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D114" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.35">
@@ -3366,10 +3366,10 @@
         <v>6</v>
       </c>
       <c r="C115" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D115" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.35">
@@ -3380,10 +3380,10 @@
         <v>7</v>
       </c>
       <c r="C116" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D116" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.35">
@@ -3394,10 +3394,10 @@
         <v>8</v>
       </c>
       <c r="C117" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D117" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.35">
@@ -3408,10 +3408,10 @@
         <v>9</v>
       </c>
       <c r="C118" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D118" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.35">
@@ -3422,10 +3422,10 @@
         <v>10</v>
       </c>
       <c r="C119" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D119" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.35">
@@ -3436,10 +3436,10 @@
         <v>11</v>
       </c>
       <c r="C120" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D120" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.35">
@@ -3450,10 +3450,10 @@
         <v>12</v>
       </c>
       <c r="C121" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D121" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.35">
@@ -3464,10 +3464,10 @@
         <v>1</v>
       </c>
       <c r="C122" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D122" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.35">
@@ -3478,10 +3478,10 @@
         <v>2</v>
       </c>
       <c r="C123" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D123" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.35">
@@ -3492,10 +3492,10 @@
         <v>3</v>
       </c>
       <c r="C124" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D124" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.35">
@@ -3506,10 +3506,10 @@
         <v>4</v>
       </c>
       <c r="C125" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D125" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.35">
@@ -3520,10 +3520,10 @@
         <v>5</v>
       </c>
       <c r="C126" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D126" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.35">
@@ -3534,10 +3534,10 @@
         <v>6</v>
       </c>
       <c r="C127" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D127" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.35">
@@ -3548,10 +3548,10 @@
         <v>7</v>
       </c>
       <c r="C128" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D128" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.35">
@@ -3562,10 +3562,10 @@
         <v>8</v>
       </c>
       <c r="C129" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D129" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.35">
@@ -3576,10 +3576,10 @@
         <v>9</v>
       </c>
       <c r="C130" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D130" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.35">
@@ -3590,10 +3590,10 @@
         <v>10</v>
       </c>
       <c r="C131" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D131" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.35">
@@ -3604,10 +3604,10 @@
         <v>11</v>
       </c>
       <c r="C132" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D132" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.35">
@@ -3618,10 +3618,10 @@
         <v>12</v>
       </c>
       <c r="C133" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D133" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.35">
@@ -3632,10 +3632,10 @@
         <v>1</v>
       </c>
       <c r="C134" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D134" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.35">
@@ -3646,10 +3646,10 @@
         <v>2</v>
       </c>
       <c r="C135" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D135" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.35">
@@ -3660,10 +3660,10 @@
         <v>3</v>
       </c>
       <c r="C136" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D136" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.35">
@@ -3674,10 +3674,10 @@
         <v>4</v>
       </c>
       <c r="C137" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D137" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.35">
@@ -3688,10 +3688,10 @@
         <v>5</v>
       </c>
       <c r="C138" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D138" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.35">
@@ -3702,10 +3702,10 @@
         <v>6</v>
       </c>
       <c r="C139" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D139" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.35">
@@ -3716,10 +3716,10 @@
         <v>7</v>
       </c>
       <c r="C140" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D140" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.35">
@@ -3730,10 +3730,10 @@
         <v>8</v>
       </c>
       <c r="C141" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D141" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.35">
@@ -3744,10 +3744,10 @@
         <v>9</v>
       </c>
       <c r="C142" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D142" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.35">
@@ -3758,10 +3758,10 @@
         <v>10</v>
       </c>
       <c r="C143" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D143" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.35">
@@ -3772,10 +3772,10 @@
         <v>11</v>
       </c>
       <c r="C144" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D144" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.35">
@@ -3786,10 +3786,10 @@
         <v>12</v>
       </c>
       <c r="C145" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D145" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.35">
@@ -3800,10 +3800,10 @@
         <v>1</v>
       </c>
       <c r="C146" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D146" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.35">
@@ -3814,10 +3814,10 @@
         <v>2</v>
       </c>
       <c r="C147" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D147" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.35">
@@ -3828,10 +3828,10 @@
         <v>3</v>
       </c>
       <c r="C148" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D148" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.35">
@@ -3842,10 +3842,10 @@
         <v>4</v>
       </c>
       <c r="C149" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D149" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.35">
@@ -3856,10 +3856,10 @@
         <v>5</v>
       </c>
       <c r="C150" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D150" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.35">
@@ -3870,10 +3870,10 @@
         <v>6</v>
       </c>
       <c r="C151" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D151" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.35">
@@ -3884,10 +3884,10 @@
         <v>7</v>
       </c>
       <c r="C152" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D152" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.35">
@@ -3898,10 +3898,10 @@
         <v>8</v>
       </c>
       <c r="C153" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D153" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.35">
@@ -3912,10 +3912,10 @@
         <v>9</v>
       </c>
       <c r="C154" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D154" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.35">
@@ -3926,10 +3926,10 @@
         <v>10</v>
       </c>
       <c r="C155" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D155" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.35">
@@ -3940,10 +3940,10 @@
         <v>11</v>
       </c>
       <c r="C156" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D156" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.35">
@@ -3954,10 +3954,10 @@
         <v>12</v>
       </c>
       <c r="C157" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D157" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.35">
@@ -3968,10 +3968,10 @@
         <v>1</v>
       </c>
       <c r="C158" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D158" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.35">
@@ -3982,10 +3982,10 @@
         <v>2</v>
       </c>
       <c r="C159" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D159" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.35">
@@ -3996,10 +3996,10 @@
         <v>3</v>
       </c>
       <c r="C160" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D160" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.35">
@@ -4010,10 +4010,10 @@
         <v>4</v>
       </c>
       <c r="C161" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D161" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.35">
@@ -4024,10 +4024,10 @@
         <v>5</v>
       </c>
       <c r="C162" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D162" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.35">
@@ -4038,10 +4038,10 @@
         <v>6</v>
       </c>
       <c r="C163" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D163" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.35">
@@ -4052,10 +4052,10 @@
         <v>7</v>
       </c>
       <c r="C164" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D164" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.35">
@@ -4066,10 +4066,10 @@
         <v>8</v>
       </c>
       <c r="C165" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D165" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.35">
@@ -4080,10 +4080,10 @@
         <v>9</v>
       </c>
       <c r="C166" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D166" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.35">
@@ -4094,10 +4094,10 @@
         <v>10</v>
       </c>
       <c r="C167" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D167" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.35">
@@ -4108,10 +4108,10 @@
         <v>11</v>
       </c>
       <c r="C168" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D168" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.35">
@@ -4122,10 +4122,10 @@
         <v>12</v>
       </c>
       <c r="C169" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D169" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.35">
@@ -4136,10 +4136,10 @@
         <v>1</v>
       </c>
       <c r="C170" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D170" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.35">
@@ -4150,10 +4150,10 @@
         <v>2</v>
       </c>
       <c r="C171" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D171" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.35">
@@ -4164,10 +4164,10 @@
         <v>3</v>
       </c>
       <c r="C172" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D172" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.35">
@@ -4178,10 +4178,10 @@
         <v>4</v>
       </c>
       <c r="C173" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D173" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.35">
@@ -4192,10 +4192,10 @@
         <v>5</v>
       </c>
       <c r="C174" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D174" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.35">
@@ -4206,10 +4206,10 @@
         <v>6</v>
       </c>
       <c r="C175" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D175" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.35">
@@ -4220,10 +4220,10 @@
         <v>7</v>
       </c>
       <c r="C176" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D176" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.35">
@@ -4234,10 +4234,10 @@
         <v>8</v>
       </c>
       <c r="C177" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D177" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.35">
@@ -4248,10 +4248,10 @@
         <v>9</v>
       </c>
       <c r="C178" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D178" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.35">
@@ -4262,10 +4262,10 @@
         <v>10</v>
       </c>
       <c r="C179" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D179" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.35">
@@ -4276,10 +4276,10 @@
         <v>11</v>
       </c>
       <c r="C180" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D180" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.35">
@@ -4290,10 +4290,10 @@
         <v>12</v>
       </c>
       <c r="C181" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D181" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.35">
@@ -4304,10 +4304,10 @@
         <v>1</v>
       </c>
       <c r="C182" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D182" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.35">
@@ -4318,10 +4318,10 @@
         <v>2</v>
       </c>
       <c r="C183" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D183" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.35">
@@ -4332,10 +4332,10 @@
         <v>3</v>
       </c>
       <c r="C184" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D184" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.35">
@@ -4346,10 +4346,10 @@
         <v>4</v>
       </c>
       <c r="C185" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D185" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.35">
@@ -4360,10 +4360,10 @@
         <v>5</v>
       </c>
       <c r="C186" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D186" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.35">
@@ -4374,10 +4374,10 @@
         <v>6</v>
       </c>
       <c r="C187" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D187" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.35">
@@ -4388,10 +4388,10 @@
         <v>7</v>
       </c>
       <c r="C188" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D188" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.35">
@@ -4402,10 +4402,10 @@
         <v>8</v>
       </c>
       <c r="C189" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D189" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.35">
@@ -4416,10 +4416,10 @@
         <v>9</v>
       </c>
       <c r="C190" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D190" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.35">
@@ -4430,10 +4430,10 @@
         <v>10</v>
       </c>
       <c r="C191" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D191" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.35">
@@ -4444,10 +4444,10 @@
         <v>11</v>
       </c>
       <c r="C192" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D192" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.35">
@@ -4458,10 +4458,10 @@
         <v>12</v>
       </c>
       <c r="C193" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D193" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.35">
@@ -4472,10 +4472,10 @@
         <v>1</v>
       </c>
       <c r="C194" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D194" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.35">
@@ -4486,10 +4486,10 @@
         <v>2</v>
       </c>
       <c r="C195" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D195" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.35">
@@ -4500,10 +4500,10 @@
         <v>3</v>
       </c>
       <c r="C196" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D196" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.35">
@@ -4514,10 +4514,10 @@
         <v>4</v>
       </c>
       <c r="C197" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D197" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.35">
@@ -4528,10 +4528,10 @@
         <v>5</v>
       </c>
       <c r="C198" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D198" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.35">
@@ -4542,10 +4542,10 @@
         <v>6</v>
       </c>
       <c r="C199" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D199" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.35">
@@ -4556,10 +4556,10 @@
         <v>7</v>
       </c>
       <c r="C200" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D200" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.35">
@@ -4570,10 +4570,10 @@
         <v>8</v>
       </c>
       <c r="C201" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D201" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.35">
@@ -4584,10 +4584,10 @@
         <v>9</v>
       </c>
       <c r="C202" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D202" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.35">
@@ -4598,10 +4598,10 @@
         <v>10</v>
       </c>
       <c r="C203" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D203" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.35">
@@ -4612,10 +4612,10 @@
         <v>11</v>
       </c>
       <c r="C204" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D204" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.35">
@@ -4626,10 +4626,10 @@
         <v>12</v>
       </c>
       <c r="C205" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D205" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.35">
@@ -4640,10 +4640,10 @@
         <v>1</v>
       </c>
       <c r="C206" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D206" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.35">
@@ -4654,10 +4654,10 @@
         <v>2</v>
       </c>
       <c r="C207" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D207" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.35">
@@ -4668,10 +4668,10 @@
         <v>3</v>
       </c>
       <c r="C208" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D208" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.35">
@@ -4682,10 +4682,10 @@
         <v>4</v>
       </c>
       <c r="C209" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D209" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.35">
@@ -4696,10 +4696,10 @@
         <v>5</v>
       </c>
       <c r="C210" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D210" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.35">
@@ -4710,10 +4710,10 @@
         <v>6</v>
       </c>
       <c r="C211" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D211" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.35">
@@ -4724,10 +4724,10 @@
         <v>7</v>
       </c>
       <c r="C212" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D212" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.35">
@@ -4738,10 +4738,10 @@
         <v>8</v>
       </c>
       <c r="C213" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D213" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.35">
@@ -4752,10 +4752,10 @@
         <v>9</v>
       </c>
       <c r="C214" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D214" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.35">
@@ -4766,10 +4766,10 @@
         <v>10</v>
       </c>
       <c r="C215" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D215" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.35">
@@ -4780,10 +4780,10 @@
         <v>11</v>
       </c>
       <c r="C216" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D216" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.35">
@@ -4794,10 +4794,10 @@
         <v>12</v>
       </c>
       <c r="C217" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D217" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.35">
@@ -4808,10 +4808,10 @@
         <v>1</v>
       </c>
       <c r="C218" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D218" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.35">
@@ -4822,10 +4822,10 @@
         <v>2</v>
       </c>
       <c r="C219" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D219" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.35">
@@ -4836,10 +4836,10 @@
         <v>3</v>
       </c>
       <c r="C220" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D220" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.35">
@@ -4850,10 +4850,10 @@
         <v>4</v>
       </c>
       <c r="C221" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D221" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.35">
@@ -4864,10 +4864,10 @@
         <v>5</v>
       </c>
       <c r="C222" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D222" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.35">
@@ -4878,10 +4878,10 @@
         <v>6</v>
       </c>
       <c r="C223" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D223" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.35">
@@ -4892,10 +4892,10 @@
         <v>7</v>
       </c>
       <c r="C224" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D224" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.35">
@@ -4906,10 +4906,10 @@
         <v>8</v>
       </c>
       <c r="C225" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D225" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.35">
@@ -4920,10 +4920,10 @@
         <v>9</v>
       </c>
       <c r="C226" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D226" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.35">
@@ -4934,10 +4934,10 @@
         <v>10</v>
       </c>
       <c r="C227" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D227" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.35">
@@ -4948,10 +4948,10 @@
         <v>11</v>
       </c>
       <c r="C228" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D228" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.35">
@@ -4962,10 +4962,10 @@
         <v>12</v>
       </c>
       <c r="C229" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D229" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.35">
@@ -4976,10 +4976,10 @@
         <v>1</v>
       </c>
       <c r="C230" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D230" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.35">
@@ -4990,10 +4990,10 @@
         <v>2</v>
       </c>
       <c r="C231" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D231" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.35">
@@ -5004,10 +5004,10 @@
         <v>3</v>
       </c>
       <c r="C232" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D232" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.35">
@@ -5018,10 +5018,10 @@
         <v>4</v>
       </c>
       <c r="C233" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D233" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.35">
@@ -5032,10 +5032,10 @@
         <v>5</v>
       </c>
       <c r="C234" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D234" s="4">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.35">
@@ -5046,10 +5046,10 @@
         <v>6</v>
       </c>
       <c r="C235" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D235" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.35">
@@ -5060,10 +5060,10 @@
         <v>7</v>
       </c>
       <c r="C236" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D236" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.35">
@@ -5074,10 +5074,10 @@
         <v>8</v>
       </c>
       <c r="C237" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D237" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.35">
@@ -5088,10 +5088,10 @@
         <v>9</v>
       </c>
       <c r="C238" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D238" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.35">
@@ -5102,10 +5102,10 @@
         <v>10</v>
       </c>
       <c r="C239" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D239" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.35">
@@ -5116,10 +5116,10 @@
         <v>11</v>
       </c>
       <c r="C240" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D240" s="4">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.35">
@@ -5130,10 +5130,10 @@
         <v>12</v>
       </c>
       <c r="C241" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D241" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Model with avalible substrate threshold
works when the conversion value is very low - adjustment to that value causes an impact on the model prematurely (repro pipeline values change drastically even before the sediment exposure spike). 

POA
-ensure export and save repro variables with every run 
-
</commit_message>
<xml_diff>
--- a/coral_data_and_custom_parameters.xlsx
+++ b/coral_data_and_custom_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10908"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katyaovsyanikova/Documents/GitHub/Coral-Model/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uqrbutto\OneDrive - The University of Queensland\PhD_proj_pollution_on_coral_reefs\Coral-Model-Rio_sediment_extension\Coral-Model-freshcopyDSenergy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C3DBF19-D95A-6948-BBE9-D1B5C3562ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3941F43C-7E7C-4CF4-959C-9904B81E0F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29700" yWindow="500" windowWidth="36860" windowHeight="18360" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Real_Cover" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Growth_Rates" sheetId="5" r:id="rId5"/>
     <sheet name="DHW_Years" sheetId="6" r:id="rId6"/>
     <sheet name="Cyclone_Years" sheetId="7" r:id="rId7"/>
+    <sheet name="Sediment_Exposure" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
   <si>
     <t>Year</t>
   </si>
@@ -97,12 +98,21 @@
   <si>
     <t>Distance_km</t>
   </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Suspended_sediment</t>
+  </si>
+  <si>
+    <t>Deposited_sediment</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -118,16 +128,60 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -150,15 +204,57 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -463,15 +559,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -485,172 +581,74 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>2000</v>
-      </c>
-      <c r="B2">
-        <v>1.2</v>
-      </c>
-      <c r="C2">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D2">
-        <v>16.3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+        <v>2012</v>
+      </c>
+      <c r="B2" s="5">
+        <v>1</v>
+      </c>
+      <c r="C2" s="9">
+        <v>2.9</v>
+      </c>
+      <c r="D2" s="5">
+        <v>5.1999999999999993</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>2001</v>
-      </c>
-      <c r="B3">
-        <v>1.55</v>
-      </c>
-      <c r="C3">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D3">
-        <v>17.399999999999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+        <v>2013</v>
+      </c>
+      <c r="B3" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="9">
+        <v>4.2</v>
+      </c>
+      <c r="D3" s="5">
+        <v>6.1000000000000005</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>2002</v>
-      </c>
-      <c r="B4">
-        <v>1.9</v>
-      </c>
-      <c r="C4">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D4">
-        <v>18.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+        <v>2014</v>
+      </c>
+      <c r="B4" s="5">
+        <v>1.7</v>
+      </c>
+      <c r="C4" s="9">
+        <v>5.4</v>
+      </c>
+      <c r="D4" s="5">
+        <v>6.7000000000000011</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>2003</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>2.4500000000000002</v>
-      </c>
-      <c r="D5">
-        <v>17.399999999999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>2015</v>
+      </c>
+      <c r="B5" s="5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9">
+        <v>8.4</v>
+      </c>
+      <c r="D5" s="5">
+        <v>3.7999999999999989</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>2004</v>
-      </c>
-      <c r="B6">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="C6">
-        <v>2.7</v>
-      </c>
-      <c r="D6">
-        <v>16.3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>2005</v>
-      </c>
-      <c r="B7">
-        <v>6.05</v>
-      </c>
-      <c r="C7">
-        <v>2.7</v>
-      </c>
-      <c r="D7">
-        <v>15.2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>2006</v>
-      </c>
-      <c r="B8">
-        <v>8</v>
-      </c>
-      <c r="C8">
-        <v>2.7</v>
-      </c>
-      <c r="D8">
-        <v>14.1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>2007</v>
-      </c>
-      <c r="B9">
-        <v>10.5</v>
-      </c>
-      <c r="C9">
-        <v>2.5499999999999998</v>
-      </c>
-      <c r="D9">
-        <v>13.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>2008</v>
-      </c>
-      <c r="B10">
-        <v>13</v>
-      </c>
-      <c r="C10">
-        <v>2.4</v>
-      </c>
-      <c r="D10">
-        <v>12.9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>2009</v>
-      </c>
-      <c r="B11">
-        <v>14.2</v>
-      </c>
-      <c r="C11">
-        <v>2.7</v>
-      </c>
-      <c r="D11">
-        <v>17.2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>2010</v>
-      </c>
-      <c r="B12">
-        <v>19.100000000000001</v>
-      </c>
-      <c r="C12">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D12">
-        <v>13.9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>2011</v>
-      </c>
-      <c r="B13">
-        <v>18.8</v>
-      </c>
-      <c r="C13">
-        <v>2.8</v>
-      </c>
-      <c r="D13">
-        <v>15.4</v>
+        <v>2016</v>
+      </c>
+      <c r="B6" s="5">
+        <v>1.5</v>
+      </c>
+      <c r="C6" s="9">
+        <v>7.6</v>
+      </c>
+      <c r="D6" s="5">
+        <v>8.5000000000000018</v>
       </c>
     </row>
   </sheetData>
@@ -661,9 +659,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -677,7 +675,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>5</v>
       </c>
@@ -691,7 +689,7 @@
         <v>7.8</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>10</v>
       </c>
@@ -705,7 +703,7 @@
         <v>10.1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>15</v>
       </c>
@@ -719,7 +717,7 @@
         <v>23.4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>20</v>
       </c>
@@ -733,7 +731,7 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>25</v>
       </c>
@@ -747,7 +745,7 @@
         <v>9.6999999999999993</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>30</v>
       </c>
@@ -761,7 +759,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>35</v>
       </c>
@@ -775,7 +773,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>40</v>
       </c>
@@ -789,7 +787,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>45</v>
       </c>
@@ -803,7 +801,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>50</v>
       </c>
@@ -817,7 +815,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>55</v>
       </c>
@@ -831,7 +829,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>60</v>
       </c>
@@ -845,7 +843,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>65</v>
       </c>
@@ -859,7 +857,7 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>70</v>
       </c>
@@ -873,7 +871,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>75</v>
       </c>
@@ -887,7 +885,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>80</v>
       </c>
@@ -901,7 +899,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>85</v>
       </c>
@@ -915,7 +913,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>90</v>
       </c>
@@ -929,7 +927,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>95</v>
       </c>
@@ -943,7 +941,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>100</v>
       </c>
@@ -965,12 +963,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -984,7 +982,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>5</v>
       </c>
@@ -998,7 +996,7 @@
         <v>1.17E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>10</v>
       </c>
@@ -1012,7 +1010,7 @@
         <v>1.3599999999999999E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>15</v>
       </c>
@@ -1026,7 +1024,7 @@
         <v>1.5599999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>20</v>
       </c>
@@ -1040,7 +1038,7 @@
         <v>1.7600000000000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>25</v>
       </c>
@@ -1054,7 +1052,7 @@
         <v>1.9599999999999999E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>30</v>
       </c>
@@ -1068,7 +1066,7 @@
         <v>2.1600000000000001E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>35</v>
       </c>
@@ -1082,7 +1080,7 @@
         <v>2.3599999999999999E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>40</v>
       </c>
@@ -1096,7 +1094,7 @@
         <v>2.5600000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>45</v>
       </c>
@@ -1110,7 +1108,7 @@
         <v>2.76E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>50</v>
       </c>
@@ -1124,7 +1122,7 @@
         <v>2.9600000000000001E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>55</v>
       </c>
@@ -1138,7 +1136,7 @@
         <v>3.1600000000000003E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>60</v>
       </c>
@@ -1152,7 +1150,7 @@
         <v>3.3500000000000002E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>65</v>
       </c>
@@ -1166,7 +1164,7 @@
         <v>3.5499999999999997E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>70</v>
       </c>
@@ -1180,7 +1178,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>75</v>
       </c>
@@ -1194,7 +1192,7 @@
         <v>3.95E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>80</v>
       </c>
@@ -1208,7 +1206,7 @@
         <v>4.1500000000000002E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>85</v>
       </c>
@@ -1222,7 +1220,7 @@
         <v>4.3499999999999997E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>90</v>
       </c>
@@ -1236,7 +1234,7 @@
         <v>4.5499999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>95</v>
       </c>
@@ -1250,7 +1248,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>100</v>
       </c>
@@ -1272,9 +1270,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1288,7 +1286,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>5</v>
       </c>
@@ -1302,7 +1300,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>10</v>
       </c>
@@ -1316,7 +1314,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>15</v>
       </c>
@@ -1330,7 +1328,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>20</v>
       </c>
@@ -1344,7 +1342,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>25</v>
       </c>
@@ -1358,7 +1356,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>30</v>
       </c>
@@ -1372,7 +1370,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>35</v>
       </c>
@@ -1386,7 +1384,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>40</v>
       </c>
@@ -1400,7 +1398,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>45</v>
       </c>
@@ -1414,7 +1412,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>50</v>
       </c>
@@ -1428,7 +1426,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>55</v>
       </c>
@@ -1442,7 +1440,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>60</v>
       </c>
@@ -1456,7 +1454,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>65</v>
       </c>
@@ -1470,7 +1468,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>70</v>
       </c>
@@ -1484,7 +1482,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>75</v>
       </c>
@@ -1498,7 +1496,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>80</v>
       </c>
@@ -1512,7 +1510,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>85</v>
       </c>
@@ -1526,7 +1524,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>90</v>
       </c>
@@ -1540,7 +1538,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>95</v>
       </c>
@@ -1554,7 +1552,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>100</v>
       </c>
@@ -1576,9 +1574,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -1586,23 +1584,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1618,9 +1616,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1628,36 +1626,36 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2013</v>
       </c>
       <c r="B2">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2016</v>
       </c>
       <c r="B3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2018</v>
       </c>
       <c r="B4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2020</v>
       </c>
       <c r="B5">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1668,9 +1666,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1681,7 +1679,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2001</v>
       </c>
@@ -1692,7 +1690,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2007</v>
       </c>
@@ -1701,6 +1699,3668 @@
       </c>
       <c r="C3">
         <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E132077E-EAF7-4017-9CD9-9B94D708D64A}">
+  <dimension ref="A1:G253"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="27" customWidth="1"/>
+    <col min="4" max="4" width="30.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="10">
+        <v>10</v>
+      </c>
+      <c r="D2" s="11">
+        <v>5</v>
+      </c>
+      <c r="G2" s="8"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2</v>
+      </c>
+      <c r="C3" s="10">
+        <v>10</v>
+      </c>
+      <c r="D3" s="11">
+        <v>5</v>
+      </c>
+      <c r="G3" s="8"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="10">
+        <v>10</v>
+      </c>
+      <c r="D4" s="11">
+        <v>5</v>
+      </c>
+      <c r="G4" s="8"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B5" s="4">
+        <v>4</v>
+      </c>
+      <c r="C5" s="10">
+        <v>10</v>
+      </c>
+      <c r="D5" s="11">
+        <v>5</v>
+      </c>
+      <c r="G5" s="8"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B6" s="4">
+        <v>5</v>
+      </c>
+      <c r="C6" s="10">
+        <v>10</v>
+      </c>
+      <c r="D6" s="11">
+        <v>5</v>
+      </c>
+      <c r="G6" s="8"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B7" s="4">
+        <v>6</v>
+      </c>
+      <c r="C7" s="10">
+        <v>10</v>
+      </c>
+      <c r="D7" s="11">
+        <v>5</v>
+      </c>
+      <c r="G7" s="8"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B8" s="4">
+        <v>7</v>
+      </c>
+      <c r="C8" s="10">
+        <v>10</v>
+      </c>
+      <c r="D8" s="11">
+        <v>5</v>
+      </c>
+      <c r="G8" s="8"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B9" s="4">
+        <v>8</v>
+      </c>
+      <c r="C9" s="10">
+        <v>10</v>
+      </c>
+      <c r="D9" s="11">
+        <v>5</v>
+      </c>
+      <c r="G9" s="8"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B10" s="4">
+        <v>9</v>
+      </c>
+      <c r="C10" s="10">
+        <v>10</v>
+      </c>
+      <c r="D10" s="11">
+        <v>5</v>
+      </c>
+      <c r="G10" s="8"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B11" s="4">
+        <v>10</v>
+      </c>
+      <c r="C11" s="10">
+        <v>10</v>
+      </c>
+      <c r="D11" s="11">
+        <v>5</v>
+      </c>
+      <c r="G11" s="8"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B12" s="4">
+        <v>11</v>
+      </c>
+      <c r="C12" s="10">
+        <v>10</v>
+      </c>
+      <c r="D12" s="11">
+        <v>5</v>
+      </c>
+      <c r="G12" s="8"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>2012</v>
+      </c>
+      <c r="B13" s="4">
+        <v>12</v>
+      </c>
+      <c r="C13" s="10">
+        <v>10</v>
+      </c>
+      <c r="D13" s="11">
+        <v>5</v>
+      </c>
+      <c r="G13" s="8"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B14" s="4">
+        <v>1</v>
+      </c>
+      <c r="C14" s="10">
+        <v>10</v>
+      </c>
+      <c r="D14" s="11">
+        <v>5</v>
+      </c>
+      <c r="G14" s="8"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B15" s="4">
+        <v>2</v>
+      </c>
+      <c r="C15" s="10">
+        <v>10</v>
+      </c>
+      <c r="D15" s="11">
+        <v>5</v>
+      </c>
+      <c r="G15" s="8"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B16" s="4">
+        <v>3</v>
+      </c>
+      <c r="C16" s="10">
+        <v>10</v>
+      </c>
+      <c r="D16" s="11">
+        <v>5</v>
+      </c>
+      <c r="G16" s="8"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B17" s="4">
+        <v>4</v>
+      </c>
+      <c r="C17" s="10">
+        <v>10</v>
+      </c>
+      <c r="D17" s="11">
+        <v>5</v>
+      </c>
+      <c r="G17" s="8"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B18" s="4">
+        <v>5</v>
+      </c>
+      <c r="C18" s="10">
+        <v>10</v>
+      </c>
+      <c r="D18" s="11">
+        <v>5</v>
+      </c>
+      <c r="G18" s="8"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B19" s="4">
+        <v>6</v>
+      </c>
+      <c r="C19" s="10">
+        <v>10</v>
+      </c>
+      <c r="D19" s="11">
+        <v>5</v>
+      </c>
+      <c r="G19" s="8"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B20" s="4">
+        <v>7</v>
+      </c>
+      <c r="C20" s="10">
+        <v>10</v>
+      </c>
+      <c r="D20" s="11">
+        <v>5</v>
+      </c>
+      <c r="G20" s="8"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B21" s="4">
+        <v>8</v>
+      </c>
+      <c r="C21" s="10">
+        <v>10</v>
+      </c>
+      <c r="D21" s="11">
+        <v>5</v>
+      </c>
+      <c r="G21" s="8"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B22" s="4">
+        <v>9</v>
+      </c>
+      <c r="C22" s="10">
+        <v>10</v>
+      </c>
+      <c r="D22" s="11">
+        <v>5</v>
+      </c>
+      <c r="G22" s="8"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B23" s="4">
+        <v>10</v>
+      </c>
+      <c r="C23" s="10">
+        <v>10</v>
+      </c>
+      <c r="D23" s="11">
+        <v>5</v>
+      </c>
+      <c r="G23" s="8"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B24" s="4">
+        <v>11</v>
+      </c>
+      <c r="C24" s="10">
+        <v>10</v>
+      </c>
+      <c r="D24" s="11">
+        <v>5</v>
+      </c>
+      <c r="G24" s="8"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
+        <v>2013</v>
+      </c>
+      <c r="B25" s="4">
+        <v>12</v>
+      </c>
+      <c r="C25" s="10">
+        <v>10</v>
+      </c>
+      <c r="D25" s="11">
+        <v>5</v>
+      </c>
+      <c r="G25" s="8"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B26" s="4">
+        <v>1</v>
+      </c>
+      <c r="C26" s="10">
+        <v>10</v>
+      </c>
+      <c r="D26" s="11">
+        <v>5</v>
+      </c>
+      <c r="G26" s="8"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B27" s="4">
+        <v>2</v>
+      </c>
+      <c r="C27" s="10">
+        <v>10</v>
+      </c>
+      <c r="D27" s="11">
+        <v>5</v>
+      </c>
+      <c r="G27" s="8"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B28" s="4">
+        <v>3</v>
+      </c>
+      <c r="C28" s="10">
+        <v>10</v>
+      </c>
+      <c r="D28" s="11">
+        <v>5</v>
+      </c>
+      <c r="G28" s="8"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B29" s="4">
+        <v>4</v>
+      </c>
+      <c r="C29" s="10">
+        <v>10</v>
+      </c>
+      <c r="D29" s="11">
+        <v>5</v>
+      </c>
+      <c r="G29" s="8"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B30" s="4">
+        <v>5</v>
+      </c>
+      <c r="C30" s="10">
+        <v>10</v>
+      </c>
+      <c r="D30" s="11">
+        <v>5</v>
+      </c>
+      <c r="G30" s="8"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B31" s="4">
+        <v>6</v>
+      </c>
+      <c r="C31" s="10">
+        <v>10</v>
+      </c>
+      <c r="D31" s="11">
+        <v>5</v>
+      </c>
+      <c r="G31" s="8"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B32" s="4">
+        <v>7</v>
+      </c>
+      <c r="C32" s="10">
+        <v>10</v>
+      </c>
+      <c r="D32" s="11">
+        <v>5</v>
+      </c>
+      <c r="G32" s="8"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B33" s="4">
+        <v>8</v>
+      </c>
+      <c r="C33" s="10">
+        <v>10</v>
+      </c>
+      <c r="D33" s="11">
+        <v>5</v>
+      </c>
+      <c r="G33" s="8"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B34" s="4">
+        <v>9</v>
+      </c>
+      <c r="C34" s="10">
+        <v>10</v>
+      </c>
+      <c r="D34" s="11">
+        <v>5</v>
+      </c>
+      <c r="G34" s="8"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B35" s="4">
+        <v>10</v>
+      </c>
+      <c r="C35" s="10">
+        <v>10</v>
+      </c>
+      <c r="D35" s="11">
+        <v>5</v>
+      </c>
+      <c r="G35" s="8"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B36" s="4">
+        <v>11</v>
+      </c>
+      <c r="C36" s="10">
+        <v>10</v>
+      </c>
+      <c r="D36" s="11">
+        <v>5</v>
+      </c>
+      <c r="G36" s="8"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="4">
+        <v>2014</v>
+      </c>
+      <c r="B37" s="4">
+        <v>12</v>
+      </c>
+      <c r="C37" s="10">
+        <v>10</v>
+      </c>
+      <c r="D37" s="11">
+        <v>5</v>
+      </c>
+      <c r="G37" s="8"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B38" s="4">
+        <v>1</v>
+      </c>
+      <c r="C38" s="10">
+        <v>10</v>
+      </c>
+      <c r="D38" s="11">
+        <v>5</v>
+      </c>
+      <c r="G38" s="8"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B39" s="4">
+        <v>2</v>
+      </c>
+      <c r="C39" s="10">
+        <v>10</v>
+      </c>
+      <c r="D39" s="11">
+        <v>5</v>
+      </c>
+      <c r="G39" s="8"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B40" s="4">
+        <v>3</v>
+      </c>
+      <c r="C40" s="10">
+        <v>10</v>
+      </c>
+      <c r="D40" s="11">
+        <v>5</v>
+      </c>
+      <c r="G40" s="8"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B41" s="4">
+        <v>4</v>
+      </c>
+      <c r="C41" s="10">
+        <v>10</v>
+      </c>
+      <c r="D41" s="11">
+        <v>5</v>
+      </c>
+      <c r="G41" s="8"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B42" s="4">
+        <v>5</v>
+      </c>
+      <c r="C42" s="10">
+        <v>10</v>
+      </c>
+      <c r="D42" s="11">
+        <v>5</v>
+      </c>
+      <c r="G42" s="8"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B43" s="4">
+        <v>6</v>
+      </c>
+      <c r="C43" s="10">
+        <v>10</v>
+      </c>
+      <c r="D43" s="11">
+        <v>5</v>
+      </c>
+      <c r="G43" s="8"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B44" s="4">
+        <v>7</v>
+      </c>
+      <c r="C44" s="10">
+        <v>10</v>
+      </c>
+      <c r="D44" s="11">
+        <v>5</v>
+      </c>
+      <c r="G44" s="8"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B45" s="4">
+        <v>8</v>
+      </c>
+      <c r="C45" s="10">
+        <v>10</v>
+      </c>
+      <c r="D45" s="11">
+        <v>5</v>
+      </c>
+      <c r="G45" s="8"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B46" s="4">
+        <v>9</v>
+      </c>
+      <c r="C46" s="10">
+        <v>10</v>
+      </c>
+      <c r="D46" s="11">
+        <v>5</v>
+      </c>
+      <c r="G46" s="8"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B47" s="4">
+        <v>10</v>
+      </c>
+      <c r="C47" s="10">
+        <v>10</v>
+      </c>
+      <c r="D47" s="11">
+        <v>5</v>
+      </c>
+      <c r="G47" s="8"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B48" s="4">
+        <v>11</v>
+      </c>
+      <c r="C48" s="10">
+        <v>10</v>
+      </c>
+      <c r="D48" s="11">
+        <v>5</v>
+      </c>
+      <c r="G48" s="8"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" s="4">
+        <v>2015</v>
+      </c>
+      <c r="B49" s="4">
+        <v>12</v>
+      </c>
+      <c r="C49" s="10">
+        <v>10</v>
+      </c>
+      <c r="D49" s="11">
+        <v>5</v>
+      </c>
+      <c r="E49" s="7"/>
+      <c r="G49" s="8"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B50" s="4">
+        <v>1</v>
+      </c>
+      <c r="C50" s="10">
+        <v>10</v>
+      </c>
+      <c r="D50" s="11">
+        <v>5</v>
+      </c>
+      <c r="E50" s="7"/>
+      <c r="G50" s="8"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B51" s="4">
+        <v>2</v>
+      </c>
+      <c r="C51" s="10">
+        <v>10</v>
+      </c>
+      <c r="D51" s="11">
+        <v>5</v>
+      </c>
+      <c r="E51" s="7"/>
+      <c r="G51" s="8"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B52" s="4">
+        <v>3</v>
+      </c>
+      <c r="C52" s="10">
+        <v>10</v>
+      </c>
+      <c r="D52" s="11">
+        <v>5</v>
+      </c>
+      <c r="E52" s="7"/>
+      <c r="G52" s="8"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A53" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B53" s="4">
+        <v>4</v>
+      </c>
+      <c r="C53" s="10">
+        <v>10</v>
+      </c>
+      <c r="D53" s="11">
+        <v>5</v>
+      </c>
+      <c r="E53" s="7"/>
+      <c r="G53" s="8"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A54" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B54" s="4">
+        <v>5</v>
+      </c>
+      <c r="C54" s="10">
+        <v>10</v>
+      </c>
+      <c r="D54" s="11">
+        <v>5</v>
+      </c>
+      <c r="E54" s="7"/>
+      <c r="G54" s="8"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B55" s="4">
+        <v>6</v>
+      </c>
+      <c r="C55" s="10">
+        <v>10</v>
+      </c>
+      <c r="D55" s="11">
+        <v>5</v>
+      </c>
+      <c r="E55" s="7"/>
+      <c r="G55" s="8"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A56" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B56" s="4">
+        <v>7</v>
+      </c>
+      <c r="C56" s="10">
+        <v>10</v>
+      </c>
+      <c r="D56" s="11">
+        <v>5</v>
+      </c>
+      <c r="E56" s="7"/>
+      <c r="G56" s="8"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A57" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B57" s="4">
+        <v>8</v>
+      </c>
+      <c r="C57" s="10">
+        <v>10</v>
+      </c>
+      <c r="D57" s="11">
+        <v>5</v>
+      </c>
+      <c r="E57" s="7"/>
+      <c r="G57" s="8"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A58" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B58" s="4">
+        <v>9</v>
+      </c>
+      <c r="C58" s="10">
+        <v>10</v>
+      </c>
+      <c r="D58" s="11">
+        <v>5</v>
+      </c>
+      <c r="E58" s="7"/>
+      <c r="G58" s="8"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A59" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B59" s="4">
+        <v>10</v>
+      </c>
+      <c r="C59" s="10">
+        <v>10</v>
+      </c>
+      <c r="D59" s="11">
+        <v>5</v>
+      </c>
+      <c r="E59" s="7"/>
+      <c r="G59" s="8"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A60" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B60" s="4">
+        <v>11</v>
+      </c>
+      <c r="C60" s="10">
+        <v>10</v>
+      </c>
+      <c r="D60" s="11">
+        <v>5</v>
+      </c>
+      <c r="E60" s="7"/>
+      <c r="G60" s="8"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A61" s="4">
+        <v>2016</v>
+      </c>
+      <c r="B61" s="4">
+        <v>12</v>
+      </c>
+      <c r="C61" s="10">
+        <v>10</v>
+      </c>
+      <c r="D61" s="11">
+        <v>5</v>
+      </c>
+      <c r="E61" s="7"/>
+      <c r="G61" s="8"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A62" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B62" s="4">
+        <v>1</v>
+      </c>
+      <c r="C62" s="10">
+        <v>10</v>
+      </c>
+      <c r="D62" s="11">
+        <v>5</v>
+      </c>
+      <c r="E62" s="7"/>
+      <c r="G62" s="8"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B63" s="4">
+        <v>2</v>
+      </c>
+      <c r="C63" s="10">
+        <v>10</v>
+      </c>
+      <c r="D63" s="11">
+        <v>5</v>
+      </c>
+      <c r="E63" s="7"/>
+      <c r="G63" s="8"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B64" s="4">
+        <v>3</v>
+      </c>
+      <c r="C64" s="10">
+        <v>10</v>
+      </c>
+      <c r="D64" s="11">
+        <v>5</v>
+      </c>
+      <c r="E64" s="7"/>
+      <c r="G64" s="8"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B65" s="4">
+        <v>4</v>
+      </c>
+      <c r="C65" s="10">
+        <v>10</v>
+      </c>
+      <c r="D65" s="11">
+        <v>5</v>
+      </c>
+      <c r="E65" s="7"/>
+      <c r="G65" s="8"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B66" s="4">
+        <v>5</v>
+      </c>
+      <c r="C66" s="10">
+        <v>10</v>
+      </c>
+      <c r="D66" s="11">
+        <v>5</v>
+      </c>
+      <c r="E66" s="7"/>
+      <c r="G66" s="8"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B67" s="4">
+        <v>6</v>
+      </c>
+      <c r="C67" s="10">
+        <v>10</v>
+      </c>
+      <c r="D67" s="11">
+        <v>5</v>
+      </c>
+      <c r="E67" s="7"/>
+      <c r="G67" s="8"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B68" s="4">
+        <v>7</v>
+      </c>
+      <c r="C68" s="10">
+        <v>10</v>
+      </c>
+      <c r="D68" s="11">
+        <v>5</v>
+      </c>
+      <c r="E68" s="7"/>
+      <c r="G68" s="8"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B69" s="4">
+        <v>8</v>
+      </c>
+      <c r="C69" s="10">
+        <v>10</v>
+      </c>
+      <c r="D69" s="11">
+        <v>5</v>
+      </c>
+      <c r="E69" s="7"/>
+      <c r="G69" s="8"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B70" s="4">
+        <v>9</v>
+      </c>
+      <c r="C70" s="10">
+        <v>10</v>
+      </c>
+      <c r="D70" s="11">
+        <v>5</v>
+      </c>
+      <c r="E70" s="7"/>
+      <c r="G70" s="8"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B71" s="4">
+        <v>10</v>
+      </c>
+      <c r="C71" s="10">
+        <v>10</v>
+      </c>
+      <c r="D71" s="11">
+        <v>5</v>
+      </c>
+      <c r="E71" s="7"/>
+      <c r="G71" s="8"/>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B72" s="4">
+        <v>11</v>
+      </c>
+      <c r="C72" s="10">
+        <v>10</v>
+      </c>
+      <c r="D72" s="11">
+        <v>5</v>
+      </c>
+      <c r="E72" s="7"/>
+      <c r="G72" s="8"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73" s="4">
+        <v>2017</v>
+      </c>
+      <c r="B73" s="4">
+        <v>12</v>
+      </c>
+      <c r="C73" s="10">
+        <v>10</v>
+      </c>
+      <c r="D73" s="11">
+        <v>5</v>
+      </c>
+      <c r="E73" s="7"/>
+      <c r="G73" s="8"/>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A74" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B74" s="4">
+        <v>1</v>
+      </c>
+      <c r="C74" s="10">
+        <v>10</v>
+      </c>
+      <c r="D74" s="11">
+        <v>5</v>
+      </c>
+      <c r="E74" s="7"/>
+      <c r="G74" s="8"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A75" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B75" s="4">
+        <v>2</v>
+      </c>
+      <c r="C75" s="10">
+        <v>10</v>
+      </c>
+      <c r="D75" s="11">
+        <v>5</v>
+      </c>
+      <c r="E75" s="7"/>
+      <c r="G75" s="8"/>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A76" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B76" s="4">
+        <v>3</v>
+      </c>
+      <c r="C76" s="10">
+        <v>10</v>
+      </c>
+      <c r="D76" s="11">
+        <v>5</v>
+      </c>
+      <c r="E76" s="7"/>
+      <c r="G76" s="8"/>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A77" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B77" s="4">
+        <v>4</v>
+      </c>
+      <c r="C77" s="10">
+        <v>10</v>
+      </c>
+      <c r="D77" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A78" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B78" s="4">
+        <v>5</v>
+      </c>
+      <c r="C78" s="10">
+        <v>10</v>
+      </c>
+      <c r="D78" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A79" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B79" s="4">
+        <v>6</v>
+      </c>
+      <c r="C79" s="10">
+        <v>10</v>
+      </c>
+      <c r="D79" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A80" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B80" s="4">
+        <v>7</v>
+      </c>
+      <c r="C80" s="10">
+        <v>10</v>
+      </c>
+      <c r="D80" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B81" s="4">
+        <v>8</v>
+      </c>
+      <c r="C81" s="10">
+        <v>10</v>
+      </c>
+      <c r="D81" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B82" s="4">
+        <v>9</v>
+      </c>
+      <c r="C82" s="10">
+        <v>10</v>
+      </c>
+      <c r="D82" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B83" s="4">
+        <v>10</v>
+      </c>
+      <c r="C83" s="10">
+        <v>10</v>
+      </c>
+      <c r="D83" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B84" s="4">
+        <v>11</v>
+      </c>
+      <c r="C84" s="10">
+        <v>10</v>
+      </c>
+      <c r="D84" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" s="4">
+        <v>2018</v>
+      </c>
+      <c r="B85" s="4">
+        <v>12</v>
+      </c>
+      <c r="C85" s="10">
+        <v>10</v>
+      </c>
+      <c r="D85" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B86" s="4">
+        <v>1</v>
+      </c>
+      <c r="C86" s="10">
+        <v>10</v>
+      </c>
+      <c r="D86" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B87" s="4">
+        <v>2</v>
+      </c>
+      <c r="C87" s="10">
+        <v>10</v>
+      </c>
+      <c r="D87" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B88" s="4">
+        <v>3</v>
+      </c>
+      <c r="C88" s="10">
+        <v>10</v>
+      </c>
+      <c r="D88" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B89" s="4">
+        <v>4</v>
+      </c>
+      <c r="C89" s="10">
+        <v>10</v>
+      </c>
+      <c r="D89" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B90" s="4">
+        <v>5</v>
+      </c>
+      <c r="C90" s="10">
+        <v>10</v>
+      </c>
+      <c r="D90" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B91" s="4">
+        <v>6</v>
+      </c>
+      <c r="C91" s="10">
+        <v>10</v>
+      </c>
+      <c r="D91" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B92" s="4">
+        <v>7</v>
+      </c>
+      <c r="C92" s="10">
+        <v>10</v>
+      </c>
+      <c r="D92" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B93" s="4">
+        <v>8</v>
+      </c>
+      <c r="C93" s="10">
+        <v>10</v>
+      </c>
+      <c r="D93" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B94" s="4">
+        <v>9</v>
+      </c>
+      <c r="C94" s="10">
+        <v>10</v>
+      </c>
+      <c r="D94" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B95" s="4">
+        <v>10</v>
+      </c>
+      <c r="C95" s="10">
+        <v>10</v>
+      </c>
+      <c r="D95" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B96" s="4">
+        <v>11</v>
+      </c>
+      <c r="C96" s="10">
+        <v>10</v>
+      </c>
+      <c r="D96" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" s="4">
+        <v>2019</v>
+      </c>
+      <c r="B97" s="4">
+        <v>12</v>
+      </c>
+      <c r="C97" s="10">
+        <v>10</v>
+      </c>
+      <c r="D97" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B98" s="4">
+        <v>1</v>
+      </c>
+      <c r="C98" s="10">
+        <v>40</v>
+      </c>
+      <c r="D98" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B99" s="4">
+        <v>2</v>
+      </c>
+      <c r="C99" s="10">
+        <v>40</v>
+      </c>
+      <c r="D99" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B100" s="4">
+        <v>3</v>
+      </c>
+      <c r="C100" s="10">
+        <v>40</v>
+      </c>
+      <c r="D100" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B101" s="4">
+        <v>4</v>
+      </c>
+      <c r="C101" s="10">
+        <v>40</v>
+      </c>
+      <c r="D101" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B102" s="4">
+        <v>5</v>
+      </c>
+      <c r="C102" s="10">
+        <v>40</v>
+      </c>
+      <c r="D102" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B103" s="4">
+        <v>6</v>
+      </c>
+      <c r="C103" s="10">
+        <v>40</v>
+      </c>
+      <c r="D103" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B104" s="4">
+        <v>7</v>
+      </c>
+      <c r="C104" s="10">
+        <v>40</v>
+      </c>
+      <c r="D104" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B105" s="4">
+        <v>8</v>
+      </c>
+      <c r="C105" s="10">
+        <v>40</v>
+      </c>
+      <c r="D105" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B106" s="4">
+        <v>9</v>
+      </c>
+      <c r="C106" s="10">
+        <v>40</v>
+      </c>
+      <c r="D106" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B107" s="4">
+        <v>10</v>
+      </c>
+      <c r="C107" s="10">
+        <v>40</v>
+      </c>
+      <c r="D107" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B108" s="4">
+        <v>11</v>
+      </c>
+      <c r="C108" s="10">
+        <v>40</v>
+      </c>
+      <c r="D108" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" s="4">
+        <v>2020</v>
+      </c>
+      <c r="B109" s="4">
+        <v>12</v>
+      </c>
+      <c r="C109" s="10">
+        <v>40</v>
+      </c>
+      <c r="D109" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B110" s="4">
+        <v>1</v>
+      </c>
+      <c r="C110" s="10">
+        <v>10</v>
+      </c>
+      <c r="D110" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B111" s="4">
+        <v>2</v>
+      </c>
+      <c r="C111" s="10">
+        <v>10</v>
+      </c>
+      <c r="D111" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B112" s="4">
+        <v>3</v>
+      </c>
+      <c r="C112" s="10">
+        <v>10</v>
+      </c>
+      <c r="D112" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B113" s="4">
+        <v>4</v>
+      </c>
+      <c r="C113" s="10">
+        <v>10</v>
+      </c>
+      <c r="D113" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B114" s="4">
+        <v>5</v>
+      </c>
+      <c r="C114" s="10">
+        <v>10</v>
+      </c>
+      <c r="D114" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B115" s="4">
+        <v>6</v>
+      </c>
+      <c r="C115" s="10">
+        <v>10</v>
+      </c>
+      <c r="D115" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B116" s="4">
+        <v>7</v>
+      </c>
+      <c r="C116" s="10">
+        <v>10</v>
+      </c>
+      <c r="D116" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B117" s="4">
+        <v>8</v>
+      </c>
+      <c r="C117" s="10">
+        <v>10</v>
+      </c>
+      <c r="D117" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B118" s="4">
+        <v>9</v>
+      </c>
+      <c r="C118" s="10">
+        <v>10</v>
+      </c>
+      <c r="D118" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B119" s="4">
+        <v>10</v>
+      </c>
+      <c r="C119" s="10">
+        <v>10</v>
+      </c>
+      <c r="D119" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A120" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B120" s="4">
+        <v>11</v>
+      </c>
+      <c r="C120" s="10">
+        <v>10</v>
+      </c>
+      <c r="D120" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A121" s="4">
+        <v>2021</v>
+      </c>
+      <c r="B121" s="4">
+        <v>12</v>
+      </c>
+      <c r="C121" s="10">
+        <v>10</v>
+      </c>
+      <c r="D121" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A122" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B122" s="4">
+        <v>1</v>
+      </c>
+      <c r="C122" s="10">
+        <v>10</v>
+      </c>
+      <c r="D122" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B123" s="4">
+        <v>2</v>
+      </c>
+      <c r="C123" s="10">
+        <v>10</v>
+      </c>
+      <c r="D123" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B124" s="4">
+        <v>3</v>
+      </c>
+      <c r="C124" s="10">
+        <v>10</v>
+      </c>
+      <c r="D124" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B125" s="4">
+        <v>4</v>
+      </c>
+      <c r="C125" s="10">
+        <v>10</v>
+      </c>
+      <c r="D125" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B126" s="4">
+        <v>5</v>
+      </c>
+      <c r="C126" s="10">
+        <v>10</v>
+      </c>
+      <c r="D126" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B127" s="4">
+        <v>6</v>
+      </c>
+      <c r="C127" s="10">
+        <v>10</v>
+      </c>
+      <c r="D127" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B128" s="4">
+        <v>7</v>
+      </c>
+      <c r="C128" s="10">
+        <v>10</v>
+      </c>
+      <c r="D128" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B129" s="4">
+        <v>8</v>
+      </c>
+      <c r="C129" s="10">
+        <v>10</v>
+      </c>
+      <c r="D129" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B130" s="4">
+        <v>9</v>
+      </c>
+      <c r="C130" s="10">
+        <v>10</v>
+      </c>
+      <c r="D130" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B131" s="4">
+        <v>10</v>
+      </c>
+      <c r="C131" s="10">
+        <v>10</v>
+      </c>
+      <c r="D131" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A132" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B132" s="4">
+        <v>11</v>
+      </c>
+      <c r="C132" s="10">
+        <v>10</v>
+      </c>
+      <c r="D132" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133" s="4">
+        <v>2022</v>
+      </c>
+      <c r="B133" s="4">
+        <v>12</v>
+      </c>
+      <c r="C133" s="10">
+        <v>10</v>
+      </c>
+      <c r="D133" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A134" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B134" s="4">
+        <v>1</v>
+      </c>
+      <c r="C134" s="10">
+        <v>10</v>
+      </c>
+      <c r="D134" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A135" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B135" s="4">
+        <v>2</v>
+      </c>
+      <c r="C135" s="10">
+        <v>10</v>
+      </c>
+      <c r="D135" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A136" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B136" s="4">
+        <v>3</v>
+      </c>
+      <c r="C136" s="10">
+        <v>10</v>
+      </c>
+      <c r="D136" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A137" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B137" s="4">
+        <v>4</v>
+      </c>
+      <c r="C137" s="10">
+        <v>10</v>
+      </c>
+      <c r="D137" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A138" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B138" s="4">
+        <v>5</v>
+      </c>
+      <c r="C138" s="10">
+        <v>10</v>
+      </c>
+      <c r="D138" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A139" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B139" s="4">
+        <v>6</v>
+      </c>
+      <c r="C139" s="10">
+        <v>10</v>
+      </c>
+      <c r="D139" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A140" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B140" s="4">
+        <v>7</v>
+      </c>
+      <c r="C140" s="10">
+        <v>10</v>
+      </c>
+      <c r="D140" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A141" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B141" s="4">
+        <v>8</v>
+      </c>
+      <c r="C141" s="10">
+        <v>10</v>
+      </c>
+      <c r="D141" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A142" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B142" s="4">
+        <v>9</v>
+      </c>
+      <c r="C142" s="10">
+        <v>10</v>
+      </c>
+      <c r="D142" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A143" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B143" s="4">
+        <v>10</v>
+      </c>
+      <c r="C143" s="10">
+        <v>10</v>
+      </c>
+      <c r="D143" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A144" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B144" s="4">
+        <v>11</v>
+      </c>
+      <c r="C144" s="10">
+        <v>10</v>
+      </c>
+      <c r="D144" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A145" s="4">
+        <v>2023</v>
+      </c>
+      <c r="B145" s="4">
+        <v>12</v>
+      </c>
+      <c r="C145" s="10">
+        <v>10</v>
+      </c>
+      <c r="D145" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A146" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B146" s="4">
+        <v>1</v>
+      </c>
+      <c r="C146" s="10">
+        <v>10</v>
+      </c>
+      <c r="D146" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A147" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B147" s="4">
+        <v>2</v>
+      </c>
+      <c r="C147" s="10">
+        <v>10</v>
+      </c>
+      <c r="D147" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A148" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B148" s="4">
+        <v>3</v>
+      </c>
+      <c r="C148" s="10">
+        <v>10</v>
+      </c>
+      <c r="D148" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A149" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B149" s="4">
+        <v>4</v>
+      </c>
+      <c r="C149" s="10">
+        <v>10</v>
+      </c>
+      <c r="D149" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A150" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B150" s="4">
+        <v>5</v>
+      </c>
+      <c r="C150" s="10">
+        <v>10</v>
+      </c>
+      <c r="D150" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A151" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B151" s="4">
+        <v>6</v>
+      </c>
+      <c r="C151" s="10">
+        <v>10</v>
+      </c>
+      <c r="D151" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A152" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B152" s="4">
+        <v>7</v>
+      </c>
+      <c r="C152" s="10">
+        <v>10</v>
+      </c>
+      <c r="D152" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A153" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B153" s="4">
+        <v>8</v>
+      </c>
+      <c r="C153" s="10">
+        <v>10</v>
+      </c>
+      <c r="D153" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A154" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B154" s="4">
+        <v>9</v>
+      </c>
+      <c r="C154" s="10">
+        <v>10</v>
+      </c>
+      <c r="D154" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A155" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B155" s="4">
+        <v>10</v>
+      </c>
+      <c r="C155" s="10">
+        <v>10</v>
+      </c>
+      <c r="D155" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A156" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B156" s="4">
+        <v>11</v>
+      </c>
+      <c r="C156" s="10">
+        <v>10</v>
+      </c>
+      <c r="D156" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A157" s="4">
+        <v>2024</v>
+      </c>
+      <c r="B157" s="4">
+        <v>12</v>
+      </c>
+      <c r="C157" s="10">
+        <v>10</v>
+      </c>
+      <c r="D157" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A158" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B158" s="4">
+        <v>1</v>
+      </c>
+      <c r="C158" s="10">
+        <v>10</v>
+      </c>
+      <c r="D158" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A159" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B159" s="4">
+        <v>2</v>
+      </c>
+      <c r="C159" s="10">
+        <v>10</v>
+      </c>
+      <c r="D159" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A160" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B160" s="4">
+        <v>3</v>
+      </c>
+      <c r="C160" s="10">
+        <v>10</v>
+      </c>
+      <c r="D160" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A161" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B161" s="4">
+        <v>4</v>
+      </c>
+      <c r="C161" s="10">
+        <v>10</v>
+      </c>
+      <c r="D161" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A162" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B162" s="4">
+        <v>5</v>
+      </c>
+      <c r="C162" s="10">
+        <v>10</v>
+      </c>
+      <c r="D162" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A163" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B163" s="4">
+        <v>6</v>
+      </c>
+      <c r="C163" s="10">
+        <v>10</v>
+      </c>
+      <c r="D163" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A164" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B164" s="4">
+        <v>7</v>
+      </c>
+      <c r="C164" s="10">
+        <v>10</v>
+      </c>
+      <c r="D164" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A165" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B165" s="4">
+        <v>8</v>
+      </c>
+      <c r="C165" s="10">
+        <v>10</v>
+      </c>
+      <c r="D165" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A166" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B166" s="4">
+        <v>9</v>
+      </c>
+      <c r="C166" s="10">
+        <v>10</v>
+      </c>
+      <c r="D166" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A167" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B167" s="4">
+        <v>10</v>
+      </c>
+      <c r="C167" s="10">
+        <v>10</v>
+      </c>
+      <c r="D167" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A168" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B168" s="4">
+        <v>11</v>
+      </c>
+      <c r="C168" s="10">
+        <v>10</v>
+      </c>
+      <c r="D168" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A169" s="4">
+        <v>2025</v>
+      </c>
+      <c r="B169" s="4">
+        <v>12</v>
+      </c>
+      <c r="C169" s="10">
+        <v>10</v>
+      </c>
+      <c r="D169" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A170" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B170" s="4">
+        <v>1</v>
+      </c>
+      <c r="C170" s="10">
+        <v>10</v>
+      </c>
+      <c r="D170" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A171" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B171" s="4">
+        <v>2</v>
+      </c>
+      <c r="C171" s="10">
+        <v>10</v>
+      </c>
+      <c r="D171" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A172" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B172" s="4">
+        <v>3</v>
+      </c>
+      <c r="C172" s="10">
+        <v>10</v>
+      </c>
+      <c r="D172" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A173" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B173" s="4">
+        <v>4</v>
+      </c>
+      <c r="C173" s="10">
+        <v>10</v>
+      </c>
+      <c r="D173" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A174" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B174" s="4">
+        <v>5</v>
+      </c>
+      <c r="C174" s="10">
+        <v>10</v>
+      </c>
+      <c r="D174" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A175" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B175" s="4">
+        <v>6</v>
+      </c>
+      <c r="C175" s="10">
+        <v>10</v>
+      </c>
+      <c r="D175" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A176" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B176" s="4">
+        <v>7</v>
+      </c>
+      <c r="C176" s="10">
+        <v>10</v>
+      </c>
+      <c r="D176" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A177" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B177" s="4">
+        <v>8</v>
+      </c>
+      <c r="C177" s="10">
+        <v>10</v>
+      </c>
+      <c r="D177" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A178" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B178" s="4">
+        <v>9</v>
+      </c>
+      <c r="C178" s="10">
+        <v>10</v>
+      </c>
+      <c r="D178" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A179" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B179" s="4">
+        <v>10</v>
+      </c>
+      <c r="C179" s="10">
+        <v>10</v>
+      </c>
+      <c r="D179" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A180" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B180" s="4">
+        <v>11</v>
+      </c>
+      <c r="C180" s="10">
+        <v>10</v>
+      </c>
+      <c r="D180" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A181" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B181" s="4">
+        <v>12</v>
+      </c>
+      <c r="C181" s="10">
+        <v>10</v>
+      </c>
+      <c r="D181" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A182" s="4">
+        <v>2027</v>
+      </c>
+      <c r="B182" s="4">
+        <v>1</v>
+      </c>
+      <c r="C182" s="10">
+        <v>10</v>
+      </c>
+      <c r="D182" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A183">
+        <v>2027</v>
+      </c>
+      <c r="B183" s="4">
+        <v>2</v>
+      </c>
+      <c r="C183" s="10">
+        <v>10</v>
+      </c>
+      <c r="D183" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A184" s="4">
+        <v>2027</v>
+      </c>
+      <c r="B184" s="4">
+        <v>3</v>
+      </c>
+      <c r="C184" s="10">
+        <v>10</v>
+      </c>
+      <c r="D184" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A185">
+        <v>2027</v>
+      </c>
+      <c r="B185" s="4">
+        <v>4</v>
+      </c>
+      <c r="C185" s="10">
+        <v>10</v>
+      </c>
+      <c r="D185" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A186" s="4">
+        <v>2027</v>
+      </c>
+      <c r="B186" s="4">
+        <v>5</v>
+      </c>
+      <c r="C186" s="10">
+        <v>10</v>
+      </c>
+      <c r="D186" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A187">
+        <v>2027</v>
+      </c>
+      <c r="B187" s="4">
+        <v>6</v>
+      </c>
+      <c r="C187" s="10">
+        <v>10</v>
+      </c>
+      <c r="D187" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A188" s="4">
+        <v>2027</v>
+      </c>
+      <c r="B188" s="4">
+        <v>7</v>
+      </c>
+      <c r="C188" s="10">
+        <v>10</v>
+      </c>
+      <c r="D188" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A189">
+        <v>2027</v>
+      </c>
+      <c r="B189" s="4">
+        <v>8</v>
+      </c>
+      <c r="C189" s="10">
+        <v>10</v>
+      </c>
+      <c r="D189" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A190" s="4">
+        <v>2027</v>
+      </c>
+      <c r="B190" s="4">
+        <v>9</v>
+      </c>
+      <c r="C190" s="10">
+        <v>10</v>
+      </c>
+      <c r="D190" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A191">
+        <v>2027</v>
+      </c>
+      <c r="B191" s="4">
+        <v>10</v>
+      </c>
+      <c r="C191" s="10">
+        <v>10</v>
+      </c>
+      <c r="D191" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A192">
+        <v>2027</v>
+      </c>
+      <c r="B192" s="4">
+        <v>11</v>
+      </c>
+      <c r="C192" s="10">
+        <v>10</v>
+      </c>
+      <c r="D192" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A193" s="4">
+        <v>2027</v>
+      </c>
+      <c r="B193" s="4">
+        <v>12</v>
+      </c>
+      <c r="C193" s="10">
+        <v>10</v>
+      </c>
+      <c r="D193" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A194">
+        <v>2028</v>
+      </c>
+      <c r="B194" s="4">
+        <v>1</v>
+      </c>
+      <c r="C194" s="10">
+        <v>10</v>
+      </c>
+      <c r="D194" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A195">
+        <v>2028</v>
+      </c>
+      <c r="B195" s="4">
+        <v>2</v>
+      </c>
+      <c r="C195" s="10">
+        <v>10</v>
+      </c>
+      <c r="D195" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A196">
+        <v>2028</v>
+      </c>
+      <c r="B196" s="4">
+        <v>3</v>
+      </c>
+      <c r="C196" s="10">
+        <v>10</v>
+      </c>
+      <c r="D196" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A197">
+        <v>2028</v>
+      </c>
+      <c r="B197" s="4">
+        <v>4</v>
+      </c>
+      <c r="C197" s="10">
+        <v>10</v>
+      </c>
+      <c r="D197" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A198">
+        <v>2028</v>
+      </c>
+      <c r="B198" s="4">
+        <v>5</v>
+      </c>
+      <c r="C198" s="10">
+        <v>10</v>
+      </c>
+      <c r="D198" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A199">
+        <v>2028</v>
+      </c>
+      <c r="B199" s="4">
+        <v>6</v>
+      </c>
+      <c r="C199" s="10">
+        <v>10</v>
+      </c>
+      <c r="D199" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A200">
+        <v>2028</v>
+      </c>
+      <c r="B200" s="4">
+        <v>7</v>
+      </c>
+      <c r="C200" s="10">
+        <v>10</v>
+      </c>
+      <c r="D200" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A201">
+        <v>2028</v>
+      </c>
+      <c r="B201" s="4">
+        <v>8</v>
+      </c>
+      <c r="C201" s="10">
+        <v>10</v>
+      </c>
+      <c r="D201" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A202">
+        <v>2028</v>
+      </c>
+      <c r="B202" s="4">
+        <v>9</v>
+      </c>
+      <c r="C202" s="10">
+        <v>10</v>
+      </c>
+      <c r="D202" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A203">
+        <v>2028</v>
+      </c>
+      <c r="B203" s="4">
+        <v>10</v>
+      </c>
+      <c r="C203" s="10">
+        <v>10</v>
+      </c>
+      <c r="D203" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A204">
+        <v>2028</v>
+      </c>
+      <c r="B204" s="4">
+        <v>11</v>
+      </c>
+      <c r="C204" s="10">
+        <v>10</v>
+      </c>
+      <c r="D204" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A205">
+        <v>2028</v>
+      </c>
+      <c r="B205" s="4">
+        <v>12</v>
+      </c>
+      <c r="C205" s="10">
+        <v>10</v>
+      </c>
+      <c r="D205" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A206">
+        <v>2029</v>
+      </c>
+      <c r="B206" s="4">
+        <v>1</v>
+      </c>
+      <c r="C206" s="10">
+        <v>10</v>
+      </c>
+      <c r="D206" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A207">
+        <v>2029</v>
+      </c>
+      <c r="B207" s="4">
+        <v>2</v>
+      </c>
+      <c r="C207" s="10">
+        <v>10</v>
+      </c>
+      <c r="D207" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A208">
+        <v>2029</v>
+      </c>
+      <c r="B208" s="4">
+        <v>3</v>
+      </c>
+      <c r="C208" s="10">
+        <v>10</v>
+      </c>
+      <c r="D208" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A209">
+        <v>2029</v>
+      </c>
+      <c r="B209" s="4">
+        <v>4</v>
+      </c>
+      <c r="C209" s="10">
+        <v>10</v>
+      </c>
+      <c r="D209" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A210">
+        <v>2029</v>
+      </c>
+      <c r="B210" s="4">
+        <v>5</v>
+      </c>
+      <c r="C210" s="10">
+        <v>10</v>
+      </c>
+      <c r="D210" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A211">
+        <v>2029</v>
+      </c>
+      <c r="B211" s="4">
+        <v>6</v>
+      </c>
+      <c r="C211" s="10">
+        <v>10</v>
+      </c>
+      <c r="D211" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A212">
+        <v>2029</v>
+      </c>
+      <c r="B212" s="4">
+        <v>7</v>
+      </c>
+      <c r="C212" s="10">
+        <v>10</v>
+      </c>
+      <c r="D212" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A213">
+        <v>2029</v>
+      </c>
+      <c r="B213" s="4">
+        <v>8</v>
+      </c>
+      <c r="C213" s="10">
+        <v>10</v>
+      </c>
+      <c r="D213" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A214">
+        <v>2029</v>
+      </c>
+      <c r="B214" s="4">
+        <v>9</v>
+      </c>
+      <c r="C214" s="10">
+        <v>10</v>
+      </c>
+      <c r="D214" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A215">
+        <v>2029</v>
+      </c>
+      <c r="B215" s="4">
+        <v>10</v>
+      </c>
+      <c r="C215" s="10">
+        <v>10</v>
+      </c>
+      <c r="D215" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A216">
+        <v>2029</v>
+      </c>
+      <c r="B216" s="4">
+        <v>11</v>
+      </c>
+      <c r="C216" s="10">
+        <v>10</v>
+      </c>
+      <c r="D216" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A217">
+        <v>2029</v>
+      </c>
+      <c r="B217" s="4">
+        <v>12</v>
+      </c>
+      <c r="C217" s="10">
+        <v>10</v>
+      </c>
+      <c r="D217" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A218">
+        <v>2030</v>
+      </c>
+      <c r="B218" s="4">
+        <v>1</v>
+      </c>
+      <c r="C218" s="10">
+        <v>10</v>
+      </c>
+      <c r="D218" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A219">
+        <v>2030</v>
+      </c>
+      <c r="B219" s="4">
+        <v>2</v>
+      </c>
+      <c r="C219" s="10">
+        <v>10</v>
+      </c>
+      <c r="D219" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A220">
+        <v>2030</v>
+      </c>
+      <c r="B220" s="4">
+        <v>3</v>
+      </c>
+      <c r="C220" s="10">
+        <v>10</v>
+      </c>
+      <c r="D220" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A221">
+        <v>2030</v>
+      </c>
+      <c r="B221" s="4">
+        <v>4</v>
+      </c>
+      <c r="C221" s="10">
+        <v>10</v>
+      </c>
+      <c r="D221" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A222">
+        <v>2030</v>
+      </c>
+      <c r="B222" s="4">
+        <v>5</v>
+      </c>
+      <c r="C222" s="10">
+        <v>10</v>
+      </c>
+      <c r="D222" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A223">
+        <v>2030</v>
+      </c>
+      <c r="B223" s="4">
+        <v>6</v>
+      </c>
+      <c r="C223" s="10">
+        <v>10</v>
+      </c>
+      <c r="D223" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A224">
+        <v>2030</v>
+      </c>
+      <c r="B224" s="4">
+        <v>7</v>
+      </c>
+      <c r="C224" s="10">
+        <v>10</v>
+      </c>
+      <c r="D224" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A225">
+        <v>2030</v>
+      </c>
+      <c r="B225" s="4">
+        <v>8</v>
+      </c>
+      <c r="C225" s="10">
+        <v>10</v>
+      </c>
+      <c r="D225" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A226">
+        <v>2030</v>
+      </c>
+      <c r="B226" s="4">
+        <v>9</v>
+      </c>
+      <c r="C226" s="10">
+        <v>10</v>
+      </c>
+      <c r="D226" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A227">
+        <v>2030</v>
+      </c>
+      <c r="B227" s="4">
+        <v>10</v>
+      </c>
+      <c r="C227" s="10">
+        <v>10</v>
+      </c>
+      <c r="D227" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A228">
+        <v>2030</v>
+      </c>
+      <c r="B228" s="4">
+        <v>11</v>
+      </c>
+      <c r="C228" s="10">
+        <v>10</v>
+      </c>
+      <c r="D228" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A229">
+        <v>2030</v>
+      </c>
+      <c r="B229" s="4">
+        <v>12</v>
+      </c>
+      <c r="C229" s="10">
+        <v>10</v>
+      </c>
+      <c r="D229" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A230">
+        <v>2031</v>
+      </c>
+      <c r="B230" s="4">
+        <v>1</v>
+      </c>
+      <c r="C230" s="10">
+        <v>10</v>
+      </c>
+      <c r="D230" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A231">
+        <v>2031</v>
+      </c>
+      <c r="B231" s="4">
+        <v>2</v>
+      </c>
+      <c r="C231" s="10">
+        <v>10</v>
+      </c>
+      <c r="D231" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A232">
+        <v>2031</v>
+      </c>
+      <c r="B232" s="4">
+        <v>3</v>
+      </c>
+      <c r="C232" s="10">
+        <v>10</v>
+      </c>
+      <c r="D232" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A233">
+        <v>2031</v>
+      </c>
+      <c r="B233" s="4">
+        <v>4</v>
+      </c>
+      <c r="C233" s="10">
+        <v>10</v>
+      </c>
+      <c r="D233" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A234">
+        <v>2031</v>
+      </c>
+      <c r="B234" s="4">
+        <v>5</v>
+      </c>
+      <c r="C234" s="10">
+        <v>10</v>
+      </c>
+      <c r="D234" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A235">
+        <v>2031</v>
+      </c>
+      <c r="B235" s="4">
+        <v>6</v>
+      </c>
+      <c r="C235" s="10">
+        <v>10</v>
+      </c>
+      <c r="D235" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A236">
+        <v>2031</v>
+      </c>
+      <c r="B236" s="4">
+        <v>7</v>
+      </c>
+      <c r="C236" s="10">
+        <v>10</v>
+      </c>
+      <c r="D236" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A237">
+        <v>2031</v>
+      </c>
+      <c r="B237" s="4">
+        <v>8</v>
+      </c>
+      <c r="C237" s="10">
+        <v>10</v>
+      </c>
+      <c r="D237" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A238">
+        <v>2031</v>
+      </c>
+      <c r="B238" s="4">
+        <v>9</v>
+      </c>
+      <c r="C238" s="10">
+        <v>10</v>
+      </c>
+      <c r="D238" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A239">
+        <v>2031</v>
+      </c>
+      <c r="B239" s="4">
+        <v>10</v>
+      </c>
+      <c r="C239" s="10">
+        <v>10</v>
+      </c>
+      <c r="D239" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="240" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A240">
+        <v>2031</v>
+      </c>
+      <c r="B240" s="4">
+        <v>11</v>
+      </c>
+      <c r="C240" s="10">
+        <v>10</v>
+      </c>
+      <c r="D240" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A241">
+        <v>2031</v>
+      </c>
+      <c r="B241" s="4">
+        <v>12</v>
+      </c>
+      <c r="C241" s="10">
+        <v>10</v>
+      </c>
+      <c r="D241" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="242" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A242">
+        <v>2032</v>
+      </c>
+      <c r="B242" s="4">
+        <v>1</v>
+      </c>
+      <c r="C242" s="10">
+        <v>10</v>
+      </c>
+      <c r="D242" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="243" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A243">
+        <v>2032</v>
+      </c>
+      <c r="B243" s="4">
+        <v>2</v>
+      </c>
+      <c r="C243" s="10">
+        <v>10</v>
+      </c>
+      <c r="D243" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A244">
+        <v>2032</v>
+      </c>
+      <c r="B244" s="4">
+        <v>3</v>
+      </c>
+      <c r="C244" s="10">
+        <v>10</v>
+      </c>
+      <c r="D244" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="245" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A245">
+        <v>2032</v>
+      </c>
+      <c r="B245" s="4">
+        <v>4</v>
+      </c>
+      <c r="C245" s="10">
+        <v>10</v>
+      </c>
+      <c r="D245" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="246" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A246">
+        <v>2032</v>
+      </c>
+      <c r="B246" s="4">
+        <v>5</v>
+      </c>
+      <c r="C246" s="10">
+        <v>10</v>
+      </c>
+      <c r="D246" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="247" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A247">
+        <v>2032</v>
+      </c>
+      <c r="B247" s="4">
+        <v>6</v>
+      </c>
+      <c r="C247" s="10">
+        <v>10</v>
+      </c>
+      <c r="D247" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="248" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A248">
+        <v>2032</v>
+      </c>
+      <c r="B248" s="4">
+        <v>7</v>
+      </c>
+      <c r="C248" s="10">
+        <v>10</v>
+      </c>
+      <c r="D248" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="249" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A249">
+        <v>2032</v>
+      </c>
+      <c r="B249" s="4">
+        <v>8</v>
+      </c>
+      <c r="C249" s="10">
+        <v>10</v>
+      </c>
+      <c r="D249" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="250" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A250">
+        <v>2032</v>
+      </c>
+      <c r="B250" s="4">
+        <v>9</v>
+      </c>
+      <c r="C250" s="10">
+        <v>10</v>
+      </c>
+      <c r="D250" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="251" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A251">
+        <v>2032</v>
+      </c>
+      <c r="B251" s="4">
+        <v>10</v>
+      </c>
+      <c r="C251" s="10">
+        <v>10</v>
+      </c>
+      <c r="D251" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="252" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A252">
+        <v>2032</v>
+      </c>
+      <c r="B252" s="4">
+        <v>11</v>
+      </c>
+      <c r="C252" s="10">
+        <v>10</v>
+      </c>
+      <c r="D252" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="253" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A253">
+        <v>2032</v>
+      </c>
+      <c r="B253" s="4">
+        <v>12</v>
+      </c>
+      <c r="C253" s="10">
+        <v>10</v>
+      </c>
+      <c r="D253" s="11">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>